<commit_message>
Added new policy creation flow
</commit_message>
<xml_diff>
--- a/kb/additional/Policies.xlsx
+++ b/kb/additional/Policies.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dr Transition\kb\additional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D84052F-0B84-43F0-AFE1-C28A668EB31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D8AAEE-B7C4-40C0-BBF8-BB9B0591CB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0A7FDD90-5045-4D28-8047-89EB9EEE2020}"/>
   </bookViews>
@@ -1802,9 +1802,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2126,766 +2125,758 @@
   <sheetFormatPr defaultColWidth="20.6328125" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>157</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>157</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>157</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>157</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>157</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>157</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>157</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>157</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>78</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>158</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>158</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" t="s">
         <v>158</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" t="s">
         <v>68</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" t="s">
         <v>158</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" t="s">
         <v>162</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" t="s">
         <v>162</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="1" t="s">
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" t="s">
         <v>162</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" t="s">
         <v>162</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" t="s">
         <v>162</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" t="s">
         <v>160</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="B22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" t="s">
         <v>23</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" t="s">
         <v>160</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" t="s">
         <v>71</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" t="s">
         <v>162</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="1" t="s">
+      <c r="A24" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" t="s">
         <v>160</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" t="s">
         <v>52</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" t="s">
         <v>160</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="B26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>52</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" t="s">
         <v>160</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" t="s">
         <v>160</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" t="s">
         <v>73</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" t="s">
         <v>160</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="1" t="s">
+      <c r="A29" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" t="s">
         <v>160</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="1" t="s">
+      <c r="A30" t="s">
         <v>41</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" t="s">
         <v>53</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" t="s">
         <v>160</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="1" t="s">
+      <c r="A31" t="s">
         <v>41</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>32</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" t="s">
         <v>54</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" t="s">
         <v>162</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>41</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="1" t="s">
+      <c r="A33" t="s">
         <v>41</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" t="s">
         <v>75</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" t="s">
         <v>160</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="1" t="s">
+      <c r="A34" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" t="s">
         <v>75</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" t="s">
         <v>160</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="1" t="s">
+      <c r="A35" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="1" t="s">
+      <c r="A36" t="s">
         <v>42</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="B36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36" t="s">
         <v>6</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" t="s">
         <v>55</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" t="s">
         <v>159</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="1" t="s">
+      <c r="A37" t="s">
         <v>43</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="1" t="s">
+      <c r="B37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" t="s">
         <v>11</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" t="s">
         <v>161</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="1" t="s">
+      <c r="A38" t="s">
         <v>43</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" t="s">
         <v>57</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" t="s">
         <v>161</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F38" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="1" t="s">
+      <c r="A39" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" t="s">
         <v>8</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" t="s">
         <v>76</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" t="s">
         <v>161</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2902,7 +2893,7 @@
       <c r="D40" t="s">
         <v>122</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" t="s">
         <v>162</v>
       </c>
       <c r="F40" t="s">
@@ -2922,7 +2913,7 @@
       <c r="D41" t="s">
         <v>123</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" t="s">
         <v>157</v>
       </c>
       <c r="F41" t="s">
@@ -2942,7 +2933,7 @@
       <c r="D42" t="s">
         <v>124</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" t="s">
         <v>157</v>
       </c>
       <c r="F42" t="s">
@@ -2962,7 +2953,7 @@
       <c r="D43" t="s">
         <v>125</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" t="s">
         <v>157</v>
       </c>
       <c r="F43" t="s">
@@ -2982,7 +2973,7 @@
       <c r="D44" t="s">
         <v>44</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" t="s">
         <v>157</v>
       </c>
       <c r="F44" t="s">
@@ -3002,7 +2993,7 @@
       <c r="D45" t="s">
         <v>45</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="E45" t="s">
         <v>157</v>
       </c>
       <c r="F45" t="s">
@@ -3022,7 +3013,7 @@
       <c r="D46" t="s">
         <v>126</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" t="s">
         <v>157</v>
       </c>
       <c r="F46" t="s">
@@ -3042,7 +3033,7 @@
       <c r="D47" t="s">
         <v>127</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E47" t="s">
         <v>157</v>
       </c>
       <c r="F47" t="s">
@@ -3062,7 +3053,7 @@
       <c r="D48" t="s">
         <v>128</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E48" t="s">
         <v>157</v>
       </c>
       <c r="F48" t="s">
@@ -3082,7 +3073,7 @@
       <c r="D49" t="s">
         <v>129</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" t="s">
         <v>162</v>
       </c>
       <c r="F49" t="s">
@@ -3116,7 +3107,7 @@
       <c r="D51" t="s">
         <v>130</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E51" t="s">
         <v>158</v>
       </c>
       <c r="F51" t="s">
@@ -3136,7 +3127,7 @@
       <c r="D52" t="s">
         <v>131</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" t="s">
         <v>158</v>
       </c>
       <c r="F52" t="s">
@@ -3156,7 +3147,7 @@
       <c r="D53" t="s">
         <v>132</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="E53" t="s">
         <v>158</v>
       </c>
       <c r="F53" t="s">
@@ -3176,7 +3167,7 @@
       <c r="D54" t="s">
         <v>133</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E54" t="s">
         <v>162</v>
       </c>
       <c r="F54" t="s">
@@ -3196,7 +3187,7 @@
       <c r="D55" t="s">
         <v>134</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" t="s">
         <v>158</v>
       </c>
       <c r="F55" t="s">
@@ -3216,7 +3207,7 @@
       <c r="D56" t="s">
         <v>135</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" t="s">
         <v>162</v>
       </c>
       <c r="F56" t="s">
@@ -3236,7 +3227,7 @@
       <c r="D57" t="s">
         <v>50</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E57" t="s">
         <v>162</v>
       </c>
       <c r="F57" t="s">
@@ -3256,7 +3247,7 @@
       <c r="D58" t="s">
         <v>136</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="E58" t="s">
         <v>162</v>
       </c>
       <c r="F58" t="s">
@@ -3276,7 +3267,7 @@
       <c r="D59" t="s">
         <v>137</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="E59" t="s">
         <v>162</v>
       </c>
       <c r="F59" t="s">
@@ -3296,7 +3287,7 @@
       <c r="D60" t="s">
         <v>138</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E60" t="s">
         <v>162</v>
       </c>
       <c r="F60" t="s">
@@ -3316,7 +3307,7 @@
       <c r="D61" t="s">
         <v>139</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" t="s">
         <v>162</v>
       </c>
       <c r="F61" t="s">
@@ -3336,7 +3327,7 @@
       <c r="D62" t="s">
         <v>140</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="E62" t="s">
         <v>162</v>
       </c>
       <c r="F62" t="s">
@@ -3356,7 +3347,7 @@
       <c r="D63" t="s">
         <v>49</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E63" t="s">
         <v>162</v>
       </c>
       <c r="F63" t="s">
@@ -3376,7 +3367,7 @@
       <c r="D64" t="s">
         <v>52</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" t="s">
         <v>160</v>
       </c>
       <c r="F64" t="s">
@@ -3396,7 +3387,7 @@
       <c r="D65" t="s">
         <v>141</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E65" t="s">
         <v>160</v>
       </c>
       <c r="F65" t="s">
@@ -3416,7 +3407,7 @@
       <c r="D66" t="s">
         <v>51</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="E66" t="s">
         <v>160</v>
       </c>
       <c r="F66" t="s">
@@ -3436,7 +3427,7 @@
       <c r="D67" t="s">
         <v>142</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E67" t="s">
         <v>160</v>
       </c>
       <c r="F67" t="s">
@@ -3456,7 +3447,7 @@
       <c r="D68" t="s">
         <v>143</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="E68" t="s">
         <v>160</v>
       </c>
       <c r="F68" t="s">
@@ -3476,7 +3467,7 @@
       <c r="D69" t="s">
         <v>144</v>
       </c>
-      <c r="E69" s="1" t="s">
+      <c r="E69" t="s">
         <v>160</v>
       </c>
       <c r="F69" t="s">
@@ -3496,7 +3487,7 @@
       <c r="D70" t="s">
         <v>145</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E70" t="s">
         <v>159</v>
       </c>
       <c r="F70" t="s">
@@ -3516,7 +3507,7 @@
       <c r="D71" t="s">
         <v>145</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="E71" t="s">
         <v>159</v>
       </c>
       <c r="F71" t="s">
@@ -3536,7 +3527,7 @@
       <c r="D72" t="s">
         <v>146</v>
       </c>
-      <c r="E72" s="1" t="s">
+      <c r="E72" t="s">
         <v>159</v>
       </c>
       <c r="F72" t="s">
@@ -3556,7 +3547,7 @@
       <c r="D73" t="s">
         <v>147</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E73" t="s">
         <v>159</v>
       </c>
       <c r="F73" t="s">
@@ -3576,7 +3567,7 @@
       <c r="D74" t="s">
         <v>145</v>
       </c>
-      <c r="E74" s="1" t="s">
+      <c r="E74" t="s">
         <v>159</v>
       </c>
       <c r="F74" t="s">
@@ -3596,7 +3587,7 @@
       <c r="D75" t="s">
         <v>148</v>
       </c>
-      <c r="E75" s="1" t="s">
+      <c r="E75" t="s">
         <v>161</v>
       </c>
       <c r="F75" t="s">
@@ -3616,7 +3607,7 @@
       <c r="D76" t="s">
         <v>149</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="E76" t="s">
         <v>161</v>
       </c>
       <c r="F76" t="s">
@@ -3636,7 +3627,7 @@
       <c r="D77" t="s">
         <v>150</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="E77" t="s">
         <v>161</v>
       </c>
       <c r="F77" t="s">
@@ -3656,7 +3647,7 @@
       <c r="D78" t="s">
         <v>151</v>
       </c>
-      <c r="E78" s="1" t="s">
+      <c r="E78" t="s">
         <v>161</v>
       </c>
       <c r="F78" t="s">
@@ -3676,7 +3667,7 @@
       <c r="D79" t="s">
         <v>152</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E79" t="s">
         <v>161</v>
       </c>
       <c r="F79" t="s">
@@ -3696,7 +3687,7 @@
       <c r="D80" t="s">
         <v>153</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="E80" t="s">
         <v>161</v>
       </c>
       <c r="F80" t="s">
@@ -3716,7 +3707,7 @@
       <c r="D81" t="s">
         <v>154</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="E81" t="s">
         <v>161</v>
       </c>
       <c r="F81" t="s">
@@ -3736,7 +3727,7 @@
       <c r="D82" t="s">
         <v>155</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E82" t="s">
         <v>161</v>
       </c>
       <c r="F82" t="s">
@@ -3744,7 +3735,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F82" xr:uid="{A7C53CE1-AB1B-4F69-8A65-C29313BFC2AD}"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{FA16102E-24DC-48CF-AC71-D68C5E17A565}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{F04BE974-3F1B-4744-A8FA-D6E3C80DFA8A}"/>

</xml_diff>

<commit_message>
Added single instance for windows Fixes
</commit_message>
<xml_diff>
--- a/kb/additional/Policies.xlsx
+++ b/kb/additional/Policies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dr Transition\kb\additional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8376E85D-52B5-4A5D-B2D9-FB4DFB4A8949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D102A468-9DD1-4A2D-A3B2-50B4570AA68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0A7FDD90-5045-4D28-8047-89EB9EEE2020}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -602,63 +602,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C32" authorId="0" shapeId="0" xr:uid="{128F4BBC-9D58-4863-B753-8777D3060594}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Filed under "Policy factsheets to adapt existing policies" in the source, but completed on the new-policy template: no "Original objective" / "Limitations" fields; "Policy description" shown under Proposed adaptations.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{CEE0D98B-BC06-4BAD-B003-448F7C4BC091}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Link seen in search results. MIT infrastructure annex to DEF 2021 (English), pending a new PGTL.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C33" authorId="0" shapeId="0" xr:uid="{F8C1AB74-2C79-4028-BBF6-35EF095C1FE7}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Filed under "Policy factsheets to adapt existing policies" in the source, but completed on the new-policy template: no "Original objective" / "Limitations" fields; "Policy description" shown under Proposed adaptations.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D33" authorId="0" shapeId="0" xr:uid="{659B61CD-38B5-45F0-A957-C73A2A78843E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>No existing policy is referenced in this factsheet (new awareness campaign).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{4B1275A2-F67B-4572-9960-A1EA3DD0589A}">
+    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{4B1275A2-F67B-4572-9960-A1EA3DD0589A}">
       <text>
         <r>
           <rPr>
@@ -672,7 +616,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{B25F87C3-E37C-4596-B732-F4AA8FE3E87A}">
+    <comment ref="D33" authorId="0" shapeId="0" xr:uid="{B25F87C3-E37C-4596-B732-F4AA8FE3E87A}">
       <text>
         <r>
           <rPr>
@@ -686,35 +630,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C36" authorId="0" shapeId="0" xr:uid="{0FB42DB6-BE7D-46BF-A572-612EFB205C01}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Filed under "Policy factsheets to adapt existing policies" in the source, but completed on the new-policy template: no "Original objective" / "Limitations" fields; "Policy description" shown under Proposed adaptations.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{9422B777-57FE-4DD6-9F45-BD1B2A5783BF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>No existing policy is referenced in this factsheet.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{A5AE8695-4927-4D14-B228-BBDF7D2CA5F4}">
+    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{A5AE8695-4927-4D14-B228-BBDF7D2CA5F4}">
       <text>
         <r>
           <rPr>
@@ -728,7 +644,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{0F80C04E-D16E-4D88-9010-0432E4FD3436}">
+    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{0F80C04E-D16E-4D88-9010-0432E4FD3436}">
       <text>
         <r>
           <rPr>
@@ -742,7 +658,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{90457D58-D5A2-4BFF-925F-DD280FFED479}">
+    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{90457D58-D5A2-4BFF-925F-DD280FFED479}">
       <text>
         <r>
           <rPr>
@@ -756,7 +672,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{DE2E0716-78AE-4DAF-B782-6F59EBF63292}">
+    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{DE2E0716-78AE-4DAF-B782-6F59EBF63292}">
       <text>
         <r>
           <rPr>
@@ -770,7 +686,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{F5FAC7D6-CC6A-42C1-85BF-0C07B000E395}">
+    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{F5FAC7D6-CC6A-42C1-85BF-0C07B000E395}">
       <text>
         <r>
           <rPr>
@@ -781,7 +697,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{A632FA71-FAA3-4976-992D-9EF4E5E18B0A}">
+    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{A632FA71-FAA3-4976-992D-9EF4E5E18B0A}">
       <text>
         <r>
           <rPr>
@@ -792,7 +708,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{D15C6D15-094B-48F6-B3CE-83EA83899870}">
+    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{D15C6D15-094B-48F6-B3CE-83EA83899870}">
       <text>
         <r>
           <rPr>
@@ -803,7 +719,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{7C6248C4-6F1B-4E76-AFFF-E9E0F8A106A7}">
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{7C6248C4-6F1B-4E76-AFFF-E9E0F8A106A7}">
       <text>
         <r>
           <rPr>
@@ -814,7 +730,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{4F270FE6-455D-475A-AF90-E3D41CF0EDB6}">
+    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{4F270FE6-455D-475A-AF90-E3D41CF0EDB6}">
       <text>
         <r>
           <rPr>
@@ -825,7 +741,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{89F84E70-4A97-4E38-A1F5-8126A7485411}">
+    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{89F84E70-4A97-4E38-A1F5-8126A7485411}">
       <text>
         <r>
           <rPr>
@@ -836,7 +752,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{280662A7-29A5-45BA-A25C-73321C94BB18}">
+    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{280662A7-29A5-45BA-A25C-73321C94BB18}">
       <text>
         <r>
           <rPr>
@@ -847,7 +763,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{C2F9E7CD-E4A6-42E7-A852-76AC8FBC95C1}">
+    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{C2F9E7CD-E4A6-42E7-A852-76AC8FBC95C1}">
       <text>
         <r>
           <rPr>
@@ -858,7 +774,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{0BA27891-D32B-413B-ACB5-8BDE169AD307}">
+    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{0BA27891-D32B-413B-ACB5-8BDE169AD307}">
       <text>
         <r>
           <rPr>
@@ -869,7 +785,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{10E51489-0262-4624-95FB-7A7493528561}">
+    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{10E51489-0262-4624-95FB-7A7493528561}">
       <text>
         <r>
           <rPr>
@@ -880,7 +796,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{94F4788C-50B8-44DF-965B-8091418C0D6B}">
+    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{94F4788C-50B8-44DF-965B-8091418C0D6B}">
       <text>
         <r>
           <rPr>
@@ -891,7 +807,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{6D7AB778-5E38-47A9-89F5-22C44BF7DDCD}">
+    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{6D7AB778-5E38-47A9-89F5-22C44BF7DDCD}">
       <text>
         <r>
           <rPr>
@@ -902,7 +818,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{86010D8A-3BEA-4CD8-A4F4-C99ED974FD9E}">
+    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{86010D8A-3BEA-4CD8-A4F4-C99ED974FD9E}">
       <text>
         <r>
           <rPr>
@@ -913,7 +829,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{91740555-7138-43AE-BD55-DCF9D57639BD}">
+    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{91740555-7138-43AE-BD55-DCF9D57639BD}">
       <text>
         <r>
           <rPr>
@@ -924,7 +840,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D55" authorId="0" shapeId="0" xr:uid="{29510604-14BD-43BE-954E-BB95DC972A75}">
+    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{29510604-14BD-43BE-954E-BB95DC972A75}">
       <text>
         <r>
           <rPr>
@@ -935,7 +851,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{51A0B6B0-FFC5-4C3E-86CF-140CB3AFB436}">
+    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{51A0B6B0-FFC5-4C3E-86CF-140CB3AFB436}">
       <text>
         <r>
           <rPr>
@@ -946,7 +862,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D57" authorId="0" shapeId="0" xr:uid="{15CB8238-AEC9-4B69-AF7C-8E0934754DEE}">
+    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{15CB8238-AEC9-4B69-AF7C-8E0934754DEE}">
       <text>
         <r>
           <rPr>
@@ -957,7 +873,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{7A2A96C3-B4FC-407E-AF23-794618E674FB}">
+    <comment ref="D55" authorId="0" shapeId="0" xr:uid="{7A2A96C3-B4FC-407E-AF23-794618E674FB}">
       <text>
         <r>
           <rPr>
@@ -968,7 +884,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{C427DF66-A7EB-4B82-90F1-A0E846EB4237}">
+    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{C427DF66-A7EB-4B82-90F1-A0E846EB4237}">
       <text>
         <r>
           <rPr>
@@ -979,7 +895,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D60" authorId="0" shapeId="0" xr:uid="{662152E2-17AB-47A3-97D7-33B0035F98B5}">
+    <comment ref="D57" authorId="0" shapeId="0" xr:uid="{662152E2-17AB-47A3-97D7-33B0035F98B5}">
       <text>
         <r>
           <rPr>
@@ -990,7 +906,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{EACBCA3C-2180-4B23-B822-8BA759744D3E}">
+    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{EACBCA3C-2180-4B23-B822-8BA759744D3E}">
       <text>
         <r>
           <rPr>
@@ -1001,7 +917,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{620DC488-411D-4173-B7A5-435D11ADA902}">
+    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{620DC488-411D-4173-B7A5-435D11ADA902}">
       <text>
         <r>
           <rPr>
@@ -1012,7 +928,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{DB12F6EB-AC19-4206-ABF1-4B90BEC67AEF}">
+    <comment ref="D60" authorId="0" shapeId="0" xr:uid="{DB12F6EB-AC19-4206-ABF1-4B90BEC67AEF}">
       <text>
         <r>
           <rPr>
@@ -1023,7 +939,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D64" authorId="0" shapeId="0" xr:uid="{E61E0C92-6990-4A34-83ED-011972D3A1A9}">
+    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{E61E0C92-6990-4A34-83ED-011972D3A1A9}">
       <text>
         <r>
           <rPr>
@@ -1034,7 +950,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D65" authorId="0" shapeId="0" xr:uid="{336FF0D6-B0F1-49C3-831E-91C277F19D39}">
+    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{336FF0D6-B0F1-49C3-831E-91C277F19D39}">
       <text>
         <r>
           <rPr>
@@ -1045,7 +961,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D66" authorId="0" shapeId="0" xr:uid="{D68A8417-5A26-416D-9919-2280443B3569}">
+    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{D68A8417-5A26-416D-9919-2280443B3569}">
       <text>
         <r>
           <rPr>
@@ -1056,7 +972,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D67" authorId="0" shapeId="0" xr:uid="{CCA3A71E-DAC3-40A7-BB94-06C0DEA5A180}">
+    <comment ref="D64" authorId="0" shapeId="0" xr:uid="{CCA3A71E-DAC3-40A7-BB94-06C0DEA5A180}">
       <text>
         <r>
           <rPr>
@@ -1067,7 +983,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D68" authorId="0" shapeId="0" xr:uid="{26635959-3244-4949-9FCA-F023FA659D8A}">
+    <comment ref="D65" authorId="0" shapeId="0" xr:uid="{26635959-3244-4949-9FCA-F023FA659D8A}">
       <text>
         <r>
           <rPr>
@@ -1078,7 +994,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D69" authorId="0" shapeId="0" xr:uid="{59826D51-C97C-48E9-9AE4-71DCD3DE2A9A}">
+    <comment ref="D66" authorId="0" shapeId="0" xr:uid="{59826D51-C97C-48E9-9AE4-71DCD3DE2A9A}">
       <text>
         <r>
           <rPr>
@@ -1089,7 +1005,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D70" authorId="0" shapeId="0" xr:uid="{E64F13D7-23E9-44AB-B844-53DE8D0A3D34}">
+    <comment ref="D67" authorId="0" shapeId="0" xr:uid="{E64F13D7-23E9-44AB-B844-53DE8D0A3D34}">
       <text>
         <r>
           <rPr>
@@ -1100,7 +1016,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{310119CF-5582-4958-A35D-19CF0F7A8C9A}">
+    <comment ref="D68" authorId="0" shapeId="0" xr:uid="{310119CF-5582-4958-A35D-19CF0F7A8C9A}">
       <text>
         <r>
           <rPr>
@@ -1111,7 +1027,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{73160079-E26A-486A-96C1-0BCE740FAD4E}">
+    <comment ref="D69" authorId="0" shapeId="0" xr:uid="{73160079-E26A-486A-96C1-0BCE740FAD4E}">
       <text>
         <r>
           <rPr>
@@ -1122,7 +1038,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D73" authorId="0" shapeId="0" xr:uid="{01751E51-B477-4058-9F90-57799D92504C}">
+    <comment ref="D70" authorId="0" shapeId="0" xr:uid="{01751E51-B477-4058-9F90-57799D92504C}">
       <text>
         <r>
           <rPr>
@@ -1133,7 +1049,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D74" authorId="0" shapeId="0" xr:uid="{EF14530C-C227-49F0-98BE-9079397A86E7}">
+    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{EF14530C-C227-49F0-98BE-9079397A86E7}">
       <text>
         <r>
           <rPr>
@@ -1144,7 +1060,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D75" authorId="0" shapeId="0" xr:uid="{915BDAC7-735F-42D4-A53B-97B55CF2EABB}">
+    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{915BDAC7-735F-42D4-A53B-97B55CF2EABB}">
       <text>
         <r>
           <rPr>
@@ -1155,7 +1071,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D76" authorId="0" shapeId="0" xr:uid="{DBB22756-EE3E-4C7D-A31E-969796B56A74}">
+    <comment ref="D73" authorId="0" shapeId="0" xr:uid="{DBB22756-EE3E-4C7D-A31E-969796B56A74}">
       <text>
         <r>
           <rPr>
@@ -1166,7 +1082,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D77" authorId="0" shapeId="0" xr:uid="{8074146F-37D2-4302-82FF-81DDB0DAB211}">
+    <comment ref="D74" authorId="0" shapeId="0" xr:uid="{8074146F-37D2-4302-82FF-81DDB0DAB211}">
       <text>
         <r>
           <rPr>
@@ -1177,7 +1093,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D78" authorId="0" shapeId="0" xr:uid="{EBDEEF43-2631-4F65-99DA-292B189FA6FE}">
+    <comment ref="D75" authorId="0" shapeId="0" xr:uid="{EBDEEF43-2631-4F65-99DA-292B189FA6FE}">
       <text>
         <r>
           <rPr>
@@ -1188,7 +1104,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D79" authorId="0" shapeId="0" xr:uid="{A71D79AE-C1B0-4D48-AEEB-7440C578B10A}">
+    <comment ref="D76" authorId="0" shapeId="0" xr:uid="{A71D79AE-C1B0-4D48-AEEB-7440C578B10A}">
       <text>
         <r>
           <rPr>
@@ -1199,7 +1115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D80" authorId="0" shapeId="0" xr:uid="{6CA170DF-AAC4-4A42-BB3C-A74F365C48D3}">
+    <comment ref="D77" authorId="0" shapeId="0" xr:uid="{6CA170DF-AAC4-4A42-BB3C-A74F365C48D3}">
       <text>
         <r>
           <rPr>
@@ -1210,7 +1126,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D81" authorId="0" shapeId="0" xr:uid="{D70111F2-3BB0-4EF4-B55D-9B20399C4F5F}">
+    <comment ref="D78" authorId="0" shapeId="0" xr:uid="{D70111F2-3BB0-4EF4-B55D-9B20399C4F5F}">
       <text>
         <r>
           <rPr>
@@ -1221,7 +1137,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D82" authorId="0" shapeId="0" xr:uid="{F335F984-A0AB-4710-B74B-4ED6A42AE180}">
+    <comment ref="D79" authorId="0" shapeId="0" xr:uid="{F335F984-A0AB-4710-B74B-4ED6A42AE180}">
       <text>
         <r>
           <rPr>
@@ -1232,7 +1148,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D83" authorId="0" shapeId="0" xr:uid="{0E2B23AE-84D2-43E3-8D81-15447DD5A08D}">
+    <comment ref="D80" authorId="0" shapeId="0" xr:uid="{0E2B23AE-84D2-43E3-8D81-15447DD5A08D}">
       <text>
         <r>
           <rPr>
@@ -1248,7 +1164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="159">
   <si>
     <t>Federal funding for energy-efficient buildings (BEG)</t>
   </si>
@@ -1262,9 +1178,6 @@
     <t>Tax relief, e.g., through adjustment of income tax (EstG)</t>
   </si>
   <si>
-    <t>Awareness campaign for policymakers and users on public transport.</t>
-  </si>
-  <si>
     <t>German Civil Code; Costs of heat supply as operating costs, regulatory authority (BGB § 556c)</t>
   </si>
   <si>
@@ -1283,9 +1196,6 @@
     <t>National Energy Poverty Strategy</t>
   </si>
   <si>
-    <t>Transport safety for women and LGBTQIA+ people</t>
-  </si>
-  <si>
     <t>Community Energy Grant</t>
   </si>
   <si>
@@ -1365,9 +1275,6 @@
   </si>
   <si>
     <t>https://docs.italia.it/media/pdf/strategia-nazionale-competenze-digitali-docs/1.0/strategia-nazionale-competenze-digitali-docs.pdf</t>
-  </si>
-  <si>
-    <t>https://mit.gov.it/nfsmitgov/files/media/pubblicazioni/2021-12/Allegato%20DEF%202021_FINALE%20230721%20FORM%20REV_ENG%203.pdf</t>
   </si>
   <si>
     <t>https://www.apren.pt/contents/legislation/decreto-legislativo-regional-17-2025-a.pdf</t>
@@ -1740,9 +1647,6 @@
   </si>
   <si>
     <t>Digital literacy policies (single platform and support for the elderly)</t>
-  </si>
-  <si>
-    <t>National Plan for Intermodal Freight Transport – Rail and Road</t>
   </si>
   <si>
     <t>Transparency on traffic rules and ZTL (Limited Traffic Zones)</t>
@@ -2111,7 +2015,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C53CE1-AB1B-4F69-8A65-C29313BFC2AD}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="20.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="100.08984375" bestFit="1" customWidth="1"/>
@@ -2119,42 +2023,42 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
         <v>43</v>
       </c>
-      <c r="B1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" t="s">
-        <v>46</v>
-      </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="D2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" t="s">
-        <v>141</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="H2">
         <f>LEN(C2)</f>
@@ -2163,46 +2067,46 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H67" si="0">LEN(C3)</f>
+        <f t="shared" ref="H3:H64" si="0">LEN(C3)</f>
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H4">
         <f t="shared" si="0"/>
@@ -2211,22 +2115,22 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
       </c>
       <c r="C5" t="s">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
@@ -2235,22 +2139,22 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
         <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
@@ -2259,22 +2163,22 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
@@ -2283,22 +2187,22 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
       <c r="C8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H8">
         <f t="shared" si="0"/>
@@ -2307,22 +2211,22 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H9">
         <f t="shared" si="0"/>
@@ -2331,22 +2235,22 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H10">
         <f t="shared" ref="H10" si="1">LEN(C10)</f>
@@ -2355,22 +2259,22 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H11">
         <f t="shared" si="0"/>
@@ -2379,22 +2283,22 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H12">
         <f t="shared" si="0"/>
@@ -2403,22 +2307,22 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E13" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H13">
         <f t="shared" si="0"/>
@@ -2427,16 +2331,16 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H14">
         <f t="shared" si="0"/>
@@ -2445,22 +2349,22 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D15" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H15">
         <f t="shared" si="0"/>
@@ -2469,22 +2373,22 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H16">
         <f t="shared" si="0"/>
@@ -2493,22 +2397,22 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E17" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H17">
         <f t="shared" si="0"/>
@@ -2517,16 +2421,16 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H18">
         <f t="shared" si="0"/>
@@ -2535,22 +2439,22 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E19" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H19">
         <f t="shared" si="0"/>
@@ -2559,22 +2463,22 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H20">
         <f t="shared" si="0"/>
@@ -2583,22 +2487,22 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H21">
         <f t="shared" si="0"/>
@@ -2607,22 +2511,22 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H22">
         <f t="shared" si="0"/>
@@ -2631,22 +2535,22 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H23">
         <f t="shared" si="0"/>
@@ -2655,22 +2559,22 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E24" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H24">
         <f t="shared" si="0"/>
@@ -2679,22 +2583,22 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E25" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H25">
         <f t="shared" si="0"/>
@@ -2703,22 +2607,22 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H26">
         <f t="shared" si="0"/>
@@ -2727,22 +2631,22 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E27" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H27">
         <f t="shared" si="0"/>
@@ -2751,22 +2655,22 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C28" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D28" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E28" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H28">
         <f t="shared" si="0"/>
@@ -2775,22 +2679,22 @@
     </row>
     <row r="29" spans="1:8" ht="15" customHeight="1">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B29" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D29" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E29" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H29">
         <f t="shared" si="0"/>
@@ -2799,22 +2703,22 @@
     </row>
     <row r="30" spans="1:8" ht="17.5" customHeight="1">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D30" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E30" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H30">
         <f t="shared" si="0"/>
@@ -2823,22 +2727,22 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C31" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E31" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H31">
         <f t="shared" si="0"/>
@@ -2847,68 +2751,74 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C32" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D32" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="E32" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H32">
         <f t="shared" si="0"/>
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C33" t="s">
-        <v>4</v>
+        <v>158</v>
+      </c>
+      <c r="D33" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" t="s">
+        <v>141</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H33">
         <f t="shared" si="0"/>
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C34" t="s">
-        <v>161</v>
+        <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="E34" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H34">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -2916,23 +2826,23 @@
         <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C35" t="s">
-        <v>162</v>
+        <v>9</v>
       </c>
       <c r="D35" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E35" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H35">
         <f t="shared" si="0"/>
-        <v>76</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2940,37 +2850,43 @@
         <v>26</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" t="s">
+        <v>142</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H36">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="E37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H37">
         <f t="shared" si="0"/>
@@ -2979,82 +2895,82 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B38" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C38" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="D38" t="s">
-        <v>41</v>
+        <v>103</v>
       </c>
       <c r="E38" t="s">
-        <v>145</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>65</v>
+        <v>143</v>
+      </c>
+      <c r="F38" t="s">
+        <v>137</v>
       </c>
       <c r="H38">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C39" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="D39" t="s">
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="E39" t="s">
-        <v>145</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>65</v>
+        <v>138</v>
+      </c>
+      <c r="F39" t="s">
+        <v>137</v>
       </c>
       <c r="H39">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C40" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="D40" t="s">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="E40" t="s">
-        <v>145</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>65</v>
+        <v>138</v>
+      </c>
+      <c r="F40" t="s">
+        <v>137</v>
       </c>
       <c r="H40">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B41" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C41" t="s">
         <v>66</v>
@@ -3063,256 +2979,256 @@
         <v>106</v>
       </c>
       <c r="E41" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="F41" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H41">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B42" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C42" t="s">
         <v>67</v>
       </c>
       <c r="D42" t="s">
-        <v>107</v>
+        <v>27</v>
       </c>
       <c r="E42" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F42" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H42">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C43" t="s">
         <v>68</v>
       </c>
       <c r="D43" t="s">
-        <v>108</v>
+        <v>28</v>
       </c>
       <c r="E43" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F43" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H43">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C44" t="s">
         <v>69</v>
       </c>
       <c r="D44" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E44" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F44" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H44">
         <f t="shared" si="0"/>
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C45" t="s">
         <v>70</v>
       </c>
       <c r="D45" t="s">
-        <v>29</v>
+        <v>108</v>
       </c>
       <c r="E45" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F45" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H45">
         <f t="shared" si="0"/>
-        <v>31</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B46" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C46" t="s">
         <v>71</v>
       </c>
       <c r="D46" t="s">
-        <v>30</v>
+        <v>109</v>
       </c>
       <c r="E46" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F46" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H46">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B47" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C47" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D47" t="s">
         <v>110</v>
       </c>
       <c r="E47" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F47" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H47">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>39</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B48" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>73</v>
-      </c>
-      <c r="D48" t="s">
-        <v>111</v>
-      </c>
-      <c r="E48" t="s">
-        <v>141</v>
+        <v>72</v>
       </c>
       <c r="F48" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H48">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C49" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D49" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E49" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F49" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H49">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>39</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B50" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C50" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="D50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E50" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H50">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B51" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C51" t="s">
         <v>75</v>
       </c>
+      <c r="D51" t="s">
+        <v>113</v>
+      </c>
+      <c r="E51" t="s">
+        <v>139</v>
+      </c>
       <c r="F51" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H51">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B52" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C52" t="s">
         <v>76</v>
@@ -3321,22 +3237,22 @@
         <v>114</v>
       </c>
       <c r="E52" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F52" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H52">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B53" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C53" t="s">
         <v>77</v>
@@ -3345,14 +3261,14 @@
         <v>115</v>
       </c>
       <c r="E53" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F53" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H53">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -3360,23 +3276,23 @@
         <v>23</v>
       </c>
       <c r="B54" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C54" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="D54" t="s">
         <v>116</v>
       </c>
       <c r="E54" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F54" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H54">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -3384,23 +3300,23 @@
         <v>23</v>
       </c>
       <c r="B55" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C55" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D55" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E55" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F55" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H55">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -3408,79 +3324,79 @@
         <v>23</v>
       </c>
       <c r="B56" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E56" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F56" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H56">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B57" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C57" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="D57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E57" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F57" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H57">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B58" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C58" t="s">
         <v>81</v>
       </c>
       <c r="D58" t="s">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="E58" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F58" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H58">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B59" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C59" t="s">
         <v>82</v>
@@ -3489,22 +3405,22 @@
         <v>120</v>
       </c>
       <c r="E59" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F59" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H59">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B60" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C60" t="s">
         <v>83</v>
@@ -3513,190 +3429,190 @@
         <v>121</v>
       </c>
       <c r="E60" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F60" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H60">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B61" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C61" t="s">
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>122</v>
+        <v>32</v>
       </c>
       <c r="E61" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H61">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B62" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C62" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="D62" t="s">
-        <v>123</v>
+        <v>35</v>
       </c>
       <c r="E62" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F62" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H62">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>39</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B63" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D63" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E63" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F63" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H63">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B64" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C64" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D64" t="s">
         <v>34</v>
       </c>
       <c r="E64" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="F64" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H64">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B65" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="D65" t="s">
-        <v>37</v>
+        <v>123</v>
       </c>
       <c r="E65" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F65" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H65">
-        <f t="shared" si="0"/>
-        <v>39</v>
+        <f t="shared" ref="H65:H80" si="2">LEN(C65)</f>
+        <v>52</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B66" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C66" t="s">
         <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E66" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F66" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H66">
-        <f t="shared" si="0"/>
-        <v>27</v>
+        <f t="shared" si="2"/>
+        <v>13</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B67" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C67" t="s">
         <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>36</v>
+        <v>125</v>
       </c>
       <c r="E67" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F67" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H67">
-        <f t="shared" si="0"/>
-        <v>38</v>
+        <f t="shared" si="2"/>
+        <v>49</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B68" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C68" t="s">
         <v>90</v>
@@ -3705,190 +3621,190 @@
         <v>126</v>
       </c>
       <c r="E68" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F68" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H68">
-        <f t="shared" ref="H68:H83" si="2">LEN(C68)</f>
-        <v>52</v>
+        <f t="shared" si="2"/>
+        <v>44</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B69" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C69" t="s">
         <v>91</v>
       </c>
       <c r="D69" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E69" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F69" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H69">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B70" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C70" t="s">
         <v>92</v>
       </c>
       <c r="D70" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E70" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F70" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H70">
         <f t="shared" si="2"/>
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B71" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C71" t="s">
         <v>93</v>
       </c>
       <c r="D71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E71" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F71" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H71">
         <f t="shared" si="2"/>
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B72" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C72" t="s">
         <v>94</v>
       </c>
       <c r="D72" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E72" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F72" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H72">
         <f t="shared" si="2"/>
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B73" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C73" t="s">
         <v>95</v>
       </c>
       <c r="D73" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E73" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F73" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H73">
         <f t="shared" si="2"/>
-        <v>34</v>
+        <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B74" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C74" t="s">
         <v>96</v>
       </c>
       <c r="D74" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E74" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F74" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H74">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B75" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C75" t="s">
         <v>97</v>
       </c>
       <c r="D75" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E75" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F75" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H75">
         <f t="shared" si="2"/>
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B76" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C76" t="s">
         <v>98</v>
@@ -3897,22 +3813,22 @@
         <v>132</v>
       </c>
       <c r="E76" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F76" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H76">
         <f t="shared" si="2"/>
-        <v>61</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B77" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C77" t="s">
         <v>99</v>
@@ -3921,22 +3837,22 @@
         <v>133</v>
       </c>
       <c r="E77" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F77" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H77">
         <f t="shared" si="2"/>
-        <v>37</v>
+        <v>11</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B78" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C78" t="s">
         <v>100</v>
@@ -3945,22 +3861,22 @@
         <v>134</v>
       </c>
       <c r="E78" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F78" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H78">
         <f t="shared" si="2"/>
-        <v>21</v>
+        <v>41</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B79" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C79" t="s">
         <v>101</v>
@@ -3969,22 +3885,22 @@
         <v>135</v>
       </c>
       <c r="E79" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F79" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H79">
         <f t="shared" si="2"/>
-        <v>24</v>
+        <v>68</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B80" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C80" t="s">
         <v>102</v>
@@ -3993,84 +3909,12 @@
         <v>136</v>
       </c>
       <c r="E80" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F80" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H80">
-        <f t="shared" si="2"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8">
-      <c r="A81" t="s">
-        <v>28</v>
-      </c>
-      <c r="B81" t="s">
-        <v>21</v>
-      </c>
-      <c r="C81" t="s">
-        <v>103</v>
-      </c>
-      <c r="D81" t="s">
-        <v>137</v>
-      </c>
-      <c r="E81" t="s">
-        <v>145</v>
-      </c>
-      <c r="F81" t="s">
-        <v>140</v>
-      </c>
-      <c r="H81">
-        <f t="shared" si="2"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8">
-      <c r="A82" t="s">
-        <v>28</v>
-      </c>
-      <c r="B82" t="s">
-        <v>21</v>
-      </c>
-      <c r="C82" t="s">
-        <v>104</v>
-      </c>
-      <c r="D82" t="s">
-        <v>138</v>
-      </c>
-      <c r="E82" t="s">
-        <v>145</v>
-      </c>
-      <c r="F82" t="s">
-        <v>140</v>
-      </c>
-      <c r="H82">
-        <f t="shared" si="2"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8">
-      <c r="A83" t="s">
-        <v>28</v>
-      </c>
-      <c r="B83" t="s">
-        <v>21</v>
-      </c>
-      <c r="C83" t="s">
-        <v>105</v>
-      </c>
-      <c r="D83" t="s">
-        <v>139</v>
-      </c>
-      <c r="E83" t="s">
-        <v>145</v>
-      </c>
-      <c r="F83" t="s">
-        <v>140</v>
-      </c>
-      <c r="H83">
         <f t="shared" si="2"/>
         <v>46</v>
       </c>
@@ -4101,61 +3945,60 @@
     <hyperlink ref="D29" r:id="rId22" xr:uid="{197D6BD6-6D24-433F-B21E-D04EE9054948}"/>
     <hyperlink ref="D30" r:id="rId23" xr:uid="{72F68369-A900-4BD1-8990-8564783A8C3C}"/>
     <hyperlink ref="D31" r:id="rId24" xr:uid="{69CD499B-1F3C-4502-99D0-575B484A534B}"/>
-    <hyperlink ref="D32" r:id="rId25" xr:uid="{7772C947-2C11-4BE4-B3AE-570EF829CB84}"/>
-    <hyperlink ref="D34" r:id="rId26" xr:uid="{6F2DAF87-0E2E-4FDB-84E9-CFDE14FFBFFF}"/>
-    <hyperlink ref="D35" r:id="rId27" xr:uid="{2CCAC871-D236-408B-B9FA-D2EB1D5E0C40}"/>
-    <hyperlink ref="D37" r:id="rId28" xr:uid="{428F6EA1-5818-4A51-BC68-3325CF77C295}"/>
-    <hyperlink ref="D38" r:id="rId29" xr:uid="{F1AFAC85-C328-421F-B5C4-2A236B4C7B84}"/>
-    <hyperlink ref="D39" r:id="rId30" xr:uid="{2929F43F-FF43-4F43-966D-B25524FC9841}"/>
-    <hyperlink ref="D40" r:id="rId31" xr:uid="{0D6A551E-F4F1-4374-9482-B1FB082B2BB4}"/>
-    <hyperlink ref="D41" r:id="rId32" xr:uid="{2756696F-298F-48A9-A14D-59F28D76A4B3}"/>
-    <hyperlink ref="D42" r:id="rId33" xr:uid="{DFA6C174-E909-4E02-97D7-ECF69BCEDC04}"/>
-    <hyperlink ref="D43" r:id="rId34" xr:uid="{42975378-F8C7-40C1-8FD9-279140112DB9}"/>
-    <hyperlink ref="D44" r:id="rId35" xr:uid="{9E861439-53A3-4E94-84A9-77B02FA0DF14}"/>
-    <hyperlink ref="D45" r:id="rId36" xr:uid="{94B7F12E-4A8A-4908-B754-CD6440105814}"/>
-    <hyperlink ref="D46" r:id="rId37" xr:uid="{D37203B1-3467-4791-97C1-D5FA4916FA26}"/>
-    <hyperlink ref="D47" r:id="rId38" xr:uid="{69F21018-CAF9-40D4-9B96-319BAB603A08}"/>
-    <hyperlink ref="D48" r:id="rId39" xr:uid="{6223FD59-6F2A-4FD8-B03E-F896BAFD2C13}"/>
-    <hyperlink ref="D49" r:id="rId40" xr:uid="{88661935-A581-4BF7-890D-E123AA21750F}"/>
-    <hyperlink ref="D50" r:id="rId41" xr:uid="{C93170FF-369B-4F8C-9D4F-3DB5C4DFF48A}"/>
-    <hyperlink ref="D52" r:id="rId42" xr:uid="{8A27131A-644F-48E1-9CB2-A067DA0D2C07}"/>
-    <hyperlink ref="D53" r:id="rId43" xr:uid="{65F1E7A9-ABA4-4FA3-8EC1-C5D350DE5FC7}"/>
-    <hyperlink ref="D54" r:id="rId44" xr:uid="{A1B0C38E-8D5F-4F6A-BE8A-B3A5C46C63F4}"/>
-    <hyperlink ref="D55" r:id="rId45" xr:uid="{4E616770-2491-4BA8-8304-F1402698BAA5}"/>
-    <hyperlink ref="D56" r:id="rId46" xr:uid="{3499484E-3B42-45C9-8CFD-55B5209AAEFB}"/>
-    <hyperlink ref="D57" r:id="rId47" xr:uid="{9587478C-75BB-4F66-AD7C-259631A01D5C}"/>
-    <hyperlink ref="D58" r:id="rId48" xr:uid="{9DB31D3B-4EF9-4EE0-8C38-17699E60A181}"/>
-    <hyperlink ref="D59" r:id="rId49" xr:uid="{B579180D-B0D5-4902-AC7E-5AAE895B8E58}"/>
-    <hyperlink ref="D60" r:id="rId50" xr:uid="{5EDACE02-0B6F-4168-B759-B80CD83049AF}"/>
-    <hyperlink ref="D61" r:id="rId51" xr:uid="{384922C9-A261-4069-8457-03FCDDC44FA2}"/>
-    <hyperlink ref="D62" r:id="rId52" xr:uid="{927A1F11-1DBA-4D32-96EE-DEA5B84C9A5D}"/>
-    <hyperlink ref="D63" r:id="rId53" xr:uid="{5D0D0DB8-AD46-4986-9B98-EAFB83433CDE}"/>
-    <hyperlink ref="D64" r:id="rId54" xr:uid="{9F0FFF7E-5E5B-4DA5-8208-87705FF0163C}"/>
-    <hyperlink ref="D65" r:id="rId55" xr:uid="{37BC9865-D94E-40FA-8D37-2EFA79072828}"/>
-    <hyperlink ref="D66" r:id="rId56" xr:uid="{913102AD-B2A9-4932-AC1D-9F71D34FBB0E}"/>
-    <hyperlink ref="D67" r:id="rId57" xr:uid="{D1CC8E83-9106-4779-B44D-BB84D924B760}"/>
-    <hyperlink ref="D68" r:id="rId58" xr:uid="{8844F135-685E-44D1-9D60-7468AD8DB244}"/>
-    <hyperlink ref="D69" r:id="rId59" xr:uid="{7B93DFA0-0E83-439A-BD2A-1414A9F63FCC}"/>
-    <hyperlink ref="D70" r:id="rId60" xr:uid="{89BFE053-4D54-4309-872E-5BEC8034683F}"/>
-    <hyperlink ref="D71" r:id="rId61" xr:uid="{D435E386-9058-438B-BA38-2873D56361D3}"/>
-    <hyperlink ref="D72" r:id="rId62" xr:uid="{9C4D4F21-640D-4DC9-952F-49248A1DBB25}"/>
-    <hyperlink ref="D73" r:id="rId63" xr:uid="{D36E8947-16AE-4484-9C63-D3E87960D04A}"/>
-    <hyperlink ref="D74" r:id="rId64" xr:uid="{F18510CB-AFA0-4AF6-8336-235F88E914E9}"/>
-    <hyperlink ref="D75" r:id="rId65" xr:uid="{7BD00D44-3373-4BFB-BFAC-64857BD433BB}"/>
-    <hyperlink ref="D76" r:id="rId66" xr:uid="{86A4FAB7-787E-49CA-A931-19A0CBAF06A8}"/>
-    <hyperlink ref="D77" r:id="rId67" xr:uid="{3AAE6721-3155-45D9-8E86-006C9F2E7837}"/>
-    <hyperlink ref="D78" r:id="rId68" xr:uid="{E33DAA04-E7BD-4CA8-8C7A-38532E177F9A}"/>
-    <hyperlink ref="D79" r:id="rId69" xr:uid="{5C3E49A6-5C26-4786-9FAB-879E0846C84D}"/>
-    <hyperlink ref="D80" r:id="rId70" xr:uid="{18540A14-49D4-4368-B1B7-DB16D1659669}"/>
-    <hyperlink ref="D81" r:id="rId71" xr:uid="{D0654701-E81D-454A-B6FF-255E627E169D}"/>
-    <hyperlink ref="D82" r:id="rId72" xr:uid="{2345F39C-F6B3-4540-900C-5E8B6C7D2510}"/>
-    <hyperlink ref="D83" r:id="rId73" xr:uid="{782EEC21-1F26-48AE-83A1-75F8799B7570}"/>
-    <hyperlink ref="D13" r:id="rId74" xr:uid="{75903415-E398-48EF-85AA-576F7EFD4BFD}"/>
-    <hyperlink ref="D12" r:id="rId75" xr:uid="{4A12E92D-D5E7-4C58-832D-CEA3CB8B359C}"/>
-    <hyperlink ref="D15" r:id="rId76" xr:uid="{B68D5E7F-5EE4-493D-980F-0F27D52CCD80}"/>
-    <hyperlink ref="D10" r:id="rId77" xr:uid="{E324A0A9-1119-4732-BCBF-35505542BD54}"/>
+    <hyperlink ref="D32" r:id="rId25" xr:uid="{6F2DAF87-0E2E-4FDB-84E9-CFDE14FFBFFF}"/>
+    <hyperlink ref="D33" r:id="rId26" xr:uid="{2CCAC871-D236-408B-B9FA-D2EB1D5E0C40}"/>
+    <hyperlink ref="D34" r:id="rId27" xr:uid="{428F6EA1-5818-4A51-BC68-3325CF77C295}"/>
+    <hyperlink ref="D35" r:id="rId28" xr:uid="{F1AFAC85-C328-421F-B5C4-2A236B4C7B84}"/>
+    <hyperlink ref="D36" r:id="rId29" xr:uid="{2929F43F-FF43-4F43-966D-B25524FC9841}"/>
+    <hyperlink ref="D37" r:id="rId30" xr:uid="{0D6A551E-F4F1-4374-9482-B1FB082B2BB4}"/>
+    <hyperlink ref="D38" r:id="rId31" xr:uid="{2756696F-298F-48A9-A14D-59F28D76A4B3}"/>
+    <hyperlink ref="D39" r:id="rId32" xr:uid="{DFA6C174-E909-4E02-97D7-ECF69BCEDC04}"/>
+    <hyperlink ref="D40" r:id="rId33" xr:uid="{42975378-F8C7-40C1-8FD9-279140112DB9}"/>
+    <hyperlink ref="D41" r:id="rId34" xr:uid="{9E861439-53A3-4E94-84A9-77B02FA0DF14}"/>
+    <hyperlink ref="D42" r:id="rId35" xr:uid="{94B7F12E-4A8A-4908-B754-CD6440105814}"/>
+    <hyperlink ref="D43" r:id="rId36" xr:uid="{D37203B1-3467-4791-97C1-D5FA4916FA26}"/>
+    <hyperlink ref="D44" r:id="rId37" xr:uid="{69F21018-CAF9-40D4-9B96-319BAB603A08}"/>
+    <hyperlink ref="D45" r:id="rId38" xr:uid="{6223FD59-6F2A-4FD8-B03E-F896BAFD2C13}"/>
+    <hyperlink ref="D46" r:id="rId39" xr:uid="{88661935-A581-4BF7-890D-E123AA21750F}"/>
+    <hyperlink ref="D47" r:id="rId40" xr:uid="{C93170FF-369B-4F8C-9D4F-3DB5C4DFF48A}"/>
+    <hyperlink ref="D49" r:id="rId41" xr:uid="{8A27131A-644F-48E1-9CB2-A067DA0D2C07}"/>
+    <hyperlink ref="D50" r:id="rId42" xr:uid="{65F1E7A9-ABA4-4FA3-8EC1-C5D350DE5FC7}"/>
+    <hyperlink ref="D51" r:id="rId43" xr:uid="{A1B0C38E-8D5F-4F6A-BE8A-B3A5C46C63F4}"/>
+    <hyperlink ref="D52" r:id="rId44" xr:uid="{4E616770-2491-4BA8-8304-F1402698BAA5}"/>
+    <hyperlink ref="D53" r:id="rId45" xr:uid="{3499484E-3B42-45C9-8CFD-55B5209AAEFB}"/>
+    <hyperlink ref="D54" r:id="rId46" xr:uid="{9587478C-75BB-4F66-AD7C-259631A01D5C}"/>
+    <hyperlink ref="D55" r:id="rId47" xr:uid="{9DB31D3B-4EF9-4EE0-8C38-17699E60A181}"/>
+    <hyperlink ref="D56" r:id="rId48" xr:uid="{B579180D-B0D5-4902-AC7E-5AAE895B8E58}"/>
+    <hyperlink ref="D57" r:id="rId49" xr:uid="{5EDACE02-0B6F-4168-B759-B80CD83049AF}"/>
+    <hyperlink ref="D58" r:id="rId50" xr:uid="{384922C9-A261-4069-8457-03FCDDC44FA2}"/>
+    <hyperlink ref="D59" r:id="rId51" xr:uid="{927A1F11-1DBA-4D32-96EE-DEA5B84C9A5D}"/>
+    <hyperlink ref="D60" r:id="rId52" xr:uid="{5D0D0DB8-AD46-4986-9B98-EAFB83433CDE}"/>
+    <hyperlink ref="D61" r:id="rId53" xr:uid="{9F0FFF7E-5E5B-4DA5-8208-87705FF0163C}"/>
+    <hyperlink ref="D62" r:id="rId54" xr:uid="{37BC9865-D94E-40FA-8D37-2EFA79072828}"/>
+    <hyperlink ref="D63" r:id="rId55" xr:uid="{913102AD-B2A9-4932-AC1D-9F71D34FBB0E}"/>
+    <hyperlink ref="D64" r:id="rId56" xr:uid="{D1CC8E83-9106-4779-B44D-BB84D924B760}"/>
+    <hyperlink ref="D65" r:id="rId57" xr:uid="{8844F135-685E-44D1-9D60-7468AD8DB244}"/>
+    <hyperlink ref="D66" r:id="rId58" xr:uid="{7B93DFA0-0E83-439A-BD2A-1414A9F63FCC}"/>
+    <hyperlink ref="D67" r:id="rId59" xr:uid="{89BFE053-4D54-4309-872E-5BEC8034683F}"/>
+    <hyperlink ref="D68" r:id="rId60" xr:uid="{D435E386-9058-438B-BA38-2873D56361D3}"/>
+    <hyperlink ref="D69" r:id="rId61" xr:uid="{9C4D4F21-640D-4DC9-952F-49248A1DBB25}"/>
+    <hyperlink ref="D70" r:id="rId62" xr:uid="{D36E8947-16AE-4484-9C63-D3E87960D04A}"/>
+    <hyperlink ref="D71" r:id="rId63" xr:uid="{F18510CB-AFA0-4AF6-8336-235F88E914E9}"/>
+    <hyperlink ref="D72" r:id="rId64" xr:uid="{7BD00D44-3373-4BFB-BFAC-64857BD433BB}"/>
+    <hyperlink ref="D73" r:id="rId65" xr:uid="{86A4FAB7-787E-49CA-A931-19A0CBAF06A8}"/>
+    <hyperlink ref="D74" r:id="rId66" xr:uid="{3AAE6721-3155-45D9-8E86-006C9F2E7837}"/>
+    <hyperlink ref="D75" r:id="rId67" xr:uid="{E33DAA04-E7BD-4CA8-8C7A-38532E177F9A}"/>
+    <hyperlink ref="D76" r:id="rId68" xr:uid="{5C3E49A6-5C26-4786-9FAB-879E0846C84D}"/>
+    <hyperlink ref="D77" r:id="rId69" xr:uid="{18540A14-49D4-4368-B1B7-DB16D1659669}"/>
+    <hyperlink ref="D78" r:id="rId70" xr:uid="{D0654701-E81D-454A-B6FF-255E627E169D}"/>
+    <hyperlink ref="D79" r:id="rId71" xr:uid="{2345F39C-F6B3-4540-900C-5E8B6C7D2510}"/>
+    <hyperlink ref="D80" r:id="rId72" xr:uid="{782EEC21-1F26-48AE-83A1-75F8799B7570}"/>
+    <hyperlink ref="D13" r:id="rId73" xr:uid="{75903415-E398-48EF-85AA-576F7EFD4BFD}"/>
+    <hyperlink ref="D12" r:id="rId74" xr:uid="{4A12E92D-D5E7-4C58-832D-CEA3CB8B359C}"/>
+    <hyperlink ref="D15" r:id="rId75" xr:uid="{B68D5E7F-5EE4-493D-980F-0F27D52CCD80}"/>
+    <hyperlink ref="D10" r:id="rId76" xr:uid="{E324A0A9-1119-4732-BCBF-35505542BD54}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId78"/>
+  <legacyDrawing r:id="rId77"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updates/fixes by 15th Oct 2026
</commit_message>
<xml_diff>
--- a/kb/additional/Policies.xlsx
+++ b/kb/additional/Policies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dr Transition\kb\additional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D102A468-9DD1-4A2D-A3B2-50B4570AA68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF1D399-81B8-4E78-A326-E329AB253DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0A7FDD90-5045-4D28-8047-89EB9EEE2020}"/>
   </bookViews>
@@ -154,7 +154,106 @@
         </r>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{4D39CDC8-7172-4B08-A80A-430CBCC6C399}">
+    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{F5FAC7D6-CC6A-42C1-85BF-0C07B000E395}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Final updated NECP 2021-2030 (Aug 2024), English. German version: same link with _de.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{A632FA71-FAA3-4976-992D-9EF4E5E18B0A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Consolidated EEG 2023 (gesetze-im-internet.de). Same URL as earlier PDF column.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{D15C6D15-094B-48F6-B3CE-83EA83899870}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Enacted law, BGBl. 2024 I Nr. 151 (in force 16.05.2024). Replaces the BMWK summary as the policy document.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{7C6248C4-6F1B-4E76-AFFF-E9E0F8A106A7}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Enacted law, BGBl. 2023 I Nr. 133 (22.05.2023). Verified scan of the same gazette: https://epflicht.ulb.uni-bonn.de/download/pdf/775275</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{4F270FE6-455D-475A-AF90-E3D41CF0EDB6}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Consolidated EnWG.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D15" authorId="0" shapeId="0" xr:uid="{89F84E70-4A97-4E38-A1F5-8126A7485411}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Consolidated text valid from 22.05.2026 (Bezirksregierung Arnsberg).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{280662A7-29A5-45BA-A25C-73321C94BB18}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Original act of 12.06.2024 (REVOSax). Note: amended 10.09.2025; consolidated HTML at revosax.sachsen.de/vorschrift/20864.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{C2F9E7CD-E4A6-42E7-A852-76AC8FBC95C1}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. NOTE: this is the NEW BüGembeteilG M-V (GVOBl. 28.04.2026) that replaced the 2016 law named in the row. No official PDF of the 2016 original was found.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{0BA27891-D32B-413B-ACB5-8BDE169AD307}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. GVBl. I Nr. 30/2019. Law repealed 28.11.2025, replaced by BbgEESG (GVBl. I Nr. 26/2025): https://www.landesrecht.brandenburg.de/dislservice/public/disl/dokumente/11224/dokument/16894</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{4D39CDC8-7172-4B08-A80A-430CBCC6C399}">
       <text>
         <r>
           <rPr>
@@ -168,7 +267,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{8D4104DA-0DC7-490A-A23A-045860D78CA0}">
+    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{8D4104DA-0DC7-490A-A23A-045860D78CA0}">
       <text>
         <r>
           <rPr>
@@ -182,7 +281,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{CC38AD26-7938-4573-9546-39F6581DB1C0}">
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{CC38AD26-7938-4573-9546-39F6581DB1C0}">
       <text>
         <r>
           <rPr>
@@ -196,7 +295,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{448474D2-CEB1-4C57-B83E-39088D6FA20D}">
+    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{448474D2-CEB1-4C57-B83E-39088D6FA20D}">
       <text>
         <r>
           <rPr>
@@ -210,7 +309,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{D9350F6B-9FDC-44DE-B0E8-B4BA96127453}">
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{D9350F6B-9FDC-44DE-B0E8-B4BA96127453}">
       <text>
         <r>
           <rPr>
@@ -224,7 +323,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{0761167D-6FCE-429A-9E21-B31176926A8A}">
+    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{0761167D-6FCE-429A-9E21-B31176926A8A}">
       <text>
         <r>
           <rPr>
@@ -238,7 +337,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{647DDD51-89ED-44B4-B15F-A9158C9DF0D7}">
+    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{647DDD51-89ED-44B4-B15F-A9158C9DF0D7}">
       <text>
         <r>
           <rPr>
@@ -252,7 +351,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{9E5054B6-C5E4-4F32-91E1-58D30F823E13}">
+    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{9E5054B6-C5E4-4F32-91E1-58D30F823E13}">
       <text>
         <r>
           <rPr>
@@ -266,7 +365,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{23149B0F-C955-46BA-A24C-FE3560D06E39}">
+    <comment ref="B24" authorId="0" shapeId="0" xr:uid="{23149B0F-C955-46BA-A24C-FE3560D06E39}">
       <text>
         <r>
           <rPr>
@@ -280,7 +379,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D15" authorId="0" shapeId="0" xr:uid="{57D59EE4-E23B-4722-A424-E8108945FB8D}">
+    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{57D59EE4-E23B-4722-A424-E8108945FB8D}">
       <text>
         <r>
           <rPr>
@@ -294,7 +393,84 @@
         </r>
       </text>
     </comment>
-    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{0C5A87B3-61E6-443C-92D6-33171E2C8AC0}">
+    <comment ref="D25" authorId="0" shapeId="0" xr:uid="{10E51489-0262-4624-95FB-7A7493528561}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Final updated NECP (Oct 2024), English. Hungarian: same link with _hu.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D26" authorId="0" shapeId="0" xr:uid="{94F4788C-50B8-44DF-965B-8091418C0D6B}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>No direct PDF of the KEHOP Plusz programme document could be found (palyazat.gov.hu serves it through a script-rendered page). Left blank rather than linking a web page.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{6D7AB778-5E38-47A9-89F5-22C44BF7DDCD}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Magyar Közlöny 2017/168 containing Govt. Decree 299/2017 (X.17.), p. 28304. Download link returns the PDF.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{86010D8A-3BEA-4CD8-A4F4-C99ED974FD9E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>NKFIH 'palyazati-felhivas' URLs serve the call PDF directly (confirmed on other NKFIH calls). Call 2020-3.1.4-ZFR-EKM.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{91740555-7138-43AE-BD55-DCF9D57639BD}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Call document, 2nd amendment (06.08.2024).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D30" authorId="0" shapeId="0" xr:uid="{29510604-14BD-43BE-954E-BB95DC972A75}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. EU BUILD UP one-stop-shop factsheet on RenoPont. RenoPont is NGO-run; no government policy document exists.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D31" authorId="0" shapeId="0" xr:uid="{51A0B6B0-FFC5-4C3E-86CF-140CB3AFB436}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Magyar Közlöny 2023/171 containing Govt. Decree 518/2023 (XI.30.), p. 9279. Housing loan scheme, not an energy policy.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{0C5A87B3-61E6-443C-92D6-33171E2C8AC0}">
       <text>
         <r>
           <rPr>
@@ -308,7 +484,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{23055DE2-2AD7-4D9C-9FFA-4ED7CFC7ADD8}">
+    <comment ref="D33" authorId="0" shapeId="0" xr:uid="{23055DE2-2AD7-4D9C-9FFA-4ED7CFC7ADD8}">
       <text>
         <r>
           <rPr>
@@ -322,7 +498,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{43D2BA42-A694-4D0F-944D-2761566385F9}">
+    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{43D2BA42-A694-4D0F-944D-2761566385F9}">
       <text>
         <r>
           <rPr>
@@ -336,7 +512,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{70BA209E-0C74-4C91-8859-AFC8EF908ED7}">
+    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{70BA209E-0C74-4C91-8859-AFC8EF908ED7}">
       <text>
         <r>
           <rPr>
@@ -350,7 +526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{54C024B5-67DB-4E8F-AAB5-D783CA6DEC8F}">
+    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{54C024B5-67DB-4E8F-AAB5-D783CA6DEC8F}">
       <text>
         <r>
           <rPr>
@@ -364,7 +540,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{B2556C7C-D3BB-49C5-9DE1-BD9CDC4DB4BC}">
+    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{B2556C7C-D3BB-49C5-9DE1-BD9CDC4DB4BC}">
       <text>
         <r>
           <rPr>
@@ -378,7 +554,95 @@
         </r>
       </text>
     </comment>
-    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{A6FA559C-8A24-47CF-83A5-96BE0812449A}">
+    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{15CB8238-AEC9-4B69-AF7C-8E0934754DEE}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Final updated NECP (July 2024).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{7A2A96C3-B4FC-407E-AF23-794618E674FB}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. CAP25 main report (latest published; CAP26 not yet out).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{C427DF66-A7EB-4B82-90F1-A0E846EB4237}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. DECC 'Micro-generation Support Scheme (MSS)' final scheme design document.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{662152E2-17AB-47A3-97D7-33B0035F98B5}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. SEAI Solar PV Grant Application Guide (scheme rules).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{EACBCA3C-2180-4B23-B822-8BA759744D3E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. SRESS 1 Application Information Pack. The separate T&amp;Cs PDF link could not be located; the pack references them.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{620DC488-411D-4173-B7A5-435D11ADA902}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Better Energy Homes Application Guide incl. Terms &amp; Conditions.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{DB12F6EB-AC19-4206-ABF1-4B90BEC67AEF}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. T&amp;Cs v2.0, Sept 2024.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{E61E0C92-6990-4A34-83ED-011972D3A1A9}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Communities Energy Grant guidelines, 2024 call.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C46" authorId="0" shapeId="0" xr:uid="{A6FA559C-8A24-47CF-83A5-96BE0812449A}">
       <text>
         <r>
           <rPr>
@@ -392,7 +656,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{26EC0D7C-508C-40F0-83B3-6DBD3AEB1E32}">
+    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{26EC0D7C-508C-40F0-83B3-6DBD3AEB1E32}">
       <text>
         <r>
           <rPr>
@@ -406,7 +670,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C23" authorId="0" shapeId="0" xr:uid="{83849BC5-8A0B-4D24-AC5D-08CC26A55C55}">
+    <comment ref="C47" authorId="0" shapeId="0" xr:uid="{83849BC5-8A0B-4D24-AC5D-08CC26A55C55}">
       <text>
         <r>
           <rPr>
@@ -420,7 +684,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{ACE66348-32A7-4127-ACB3-7BB28F057EBC}">
+    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{ACE66348-32A7-4127-ACB3-7BB28F057EBC}">
       <text>
         <r>
           <rPr>
@@ -434,7 +698,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C24" authorId="0" shapeId="0" xr:uid="{03A9D88E-4198-4085-9304-3033B3A05067}">
+    <comment ref="C48" authorId="0" shapeId="0" xr:uid="{03A9D88E-4198-4085-9304-3033B3A05067}">
       <text>
         <r>
           <rPr>
@@ -448,7 +712,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{DA744152-999B-4C4E-A7D7-7EC46B40601F}">
+    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{DA744152-999B-4C4E-A7D7-7EC46B40601F}">
       <text>
         <r>
           <rPr>
@@ -462,7 +726,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{4A3E2F7F-5EAF-4285-B201-A740B8DC6B62}">
+    <comment ref="C49" authorId="0" shapeId="0" xr:uid="{4A3E2F7F-5EAF-4285-B201-A740B8DC6B62}">
       <text>
         <r>
           <rPr>
@@ -476,7 +740,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D25" authorId="0" shapeId="0" xr:uid="{41E92815-67EB-40DB-A1FE-21BBD4A1C3D5}">
+    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{41E92815-67EB-40DB-A1FE-21BBD4A1C3D5}">
       <text>
         <r>
           <rPr>
@@ -490,7 +754,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C26" authorId="0" shapeId="0" xr:uid="{DDBC2F79-D55A-42FB-AC01-8201191DAF43}">
+    <comment ref="C50" authorId="0" shapeId="0" xr:uid="{DDBC2F79-D55A-42FB-AC01-8201191DAF43}">
       <text>
         <r>
           <rPr>
@@ -504,7 +768,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D26" authorId="0" shapeId="0" xr:uid="{4D6F3EDD-1CA9-4A80-8AD5-A6A74CD1869F}">
+    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{4D6F3EDD-1CA9-4A80-8AD5-A6A74CD1869F}">
       <text>
         <r>
           <rPr>
@@ -518,7 +782,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C27" authorId="0" shapeId="0" xr:uid="{333B9BC9-BA11-4610-A8D7-50C91C291AE9}">
+    <comment ref="C51" authorId="0" shapeId="0" xr:uid="{333B9BC9-BA11-4610-A8D7-50C91C291AE9}">
       <text>
         <r>
           <rPr>
@@ -532,7 +796,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{7DCACA42-AC3C-4F0B-8CC6-D59CEBE56563}">
+    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{7DCACA42-AC3C-4F0B-8CC6-D59CEBE56563}">
       <text>
         <r>
           <rPr>
@@ -546,7 +810,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{C61C3A1F-B3A6-4C26-9DB6-6F1CC1656B68}">
+    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{C61C3A1F-B3A6-4C26-9DB6-6F1CC1656B68}">
       <text>
         <r>
           <rPr>
@@ -560,7 +824,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{3F49A8D3-DDB8-44CF-AD99-6F26DA8532BC}">
+    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{3F49A8D3-DDB8-44CF-AD99-6F26DA8532BC}">
       <text>
         <r>
           <rPr>
@@ -574,7 +838,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D30" authorId="0" shapeId="0" xr:uid="{AE5C7866-BB1A-4E14-B1D3-9816BB5DB524}">
+    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{AE5C7866-BB1A-4E14-B1D3-9816BB5DB524}">
       <text>
         <r>
           <rPr>
@@ -588,7 +852,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D31" authorId="0" shapeId="0" xr:uid="{21CACC92-85D7-4ADA-B06D-499830F2F44F}">
+    <comment ref="D55" authorId="0" shapeId="0" xr:uid="{21CACC92-85D7-4ADA-B06D-499830F2F44F}">
       <text>
         <r>
           <rPr>
@@ -602,7 +866,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{4B1275A2-F67B-4572-9960-A1EA3DD0589A}">
+    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{4B1275A2-F67B-4572-9960-A1EA3DD0589A}">
       <text>
         <r>
           <rPr>
@@ -616,7 +880,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D33" authorId="0" shapeId="0" xr:uid="{B25F87C3-E37C-4596-B732-F4AA8FE3E87A}">
+    <comment ref="D57" authorId="0" shapeId="0" xr:uid="{B25F87C3-E37C-4596-B732-F4AA8FE3E87A}">
       <text>
         <r>
           <rPr>
@@ -630,7 +894,73 @@
         </r>
       </text>
     </comment>
-    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{A5AE8695-4927-4D14-B228-BBDF7D2CA5F4}">
+    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{336FF0D6-B0F1-49C3-831E-91C277F19D39}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>PNIEC 2024 final (MASE). Same URL as earlier PDF column.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{D68A8417-5A26-416D-9919-2280443B3569}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. GU n.285 of 30.11.2021, S.O. n.42 (original text). Consolidated copy (non-official host): https://faolex.fao.org/docs/pdf/ita227896.pdf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D60" authorId="0" shapeId="0" xr:uid="{CCA3A71E-DAC3-40A7-BB94-06C0DEA5A180}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>MASE document-library link that serves the PDF of DM 7.12.2023 n.414 (CACER decree), published 23.01.2024.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{26635959-3244-4949-9FCA-F023FA659D8A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>MASE document-library PDF: CACER Operational Rules (July 2025) governing the PNRR 40% grant.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{59826D51-C97C-48E9-9AE4-71DCD3DE2A9A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Ordinanza n.24 of 30.06.2022 approving the CER call.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{E64F13D7-23E9-44AB-B844-53DE8D0A3D34}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Representative: Piedmont Regional Law 12/2018 (first regional CER law).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D64" authorId="0" shapeId="0" xr:uid="{A5AE8695-4927-4D14-B228-BBDF7D2CA5F4}">
       <text>
         <r>
           <rPr>
@@ -644,7 +974,62 @@
         </r>
       </text>
     </comment>
-    <comment ref="D35" authorId="0" shapeId="0" xr:uid="{0F80C04E-D16E-4D88-9010-0432E4FD3436}">
+    <comment ref="D65" authorId="0" shapeId="0" xr:uid="{310119CF-5582-4958-A35D-19CF0F7A8C9A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 as published (DR 1st series n.10, pp.3-185). A copy of the same file is at https://ordemdosengenheiros.pt/fotos/especialidades/0000300185_19938915836571aac8a132c.pdf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D66" authorId="0" shapeId="0" xr:uid="{73160079-E26A-486A-96C1-0BCE740FAD4E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 (energy communities incl. cooperative form). Same document as REC framework row.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D67" authorId="0" shapeId="0" xr:uid="{01751E51-B477-4058-9F90-57799D92504C}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Regulation of the Programa de Apoio a Edifícios Mais Sustentáveis (Despacho 8745/2020). NON-OFFICIAL host (municipality); the official DR PDF could not be located.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D68" authorId="0" shapeId="0" xr:uid="{EF14530C-C227-49F0-98BE-9079397A86E7}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Direct PDF link found in search results. Lei 12/2022 (State Budget 2022) that added item 2.37 to VAT List I. Reportedly expired 30.06.2025.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D69" authorId="0" shapeId="0" xr:uid="{915BDAC7-735F-42D4-A53B-97B55CF2EABB}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 (self-consumption/UPAC rules). Same document as REC framework row.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D70" authorId="0" shapeId="0" xr:uid="{0F80C04E-D16E-4D88-9010-0432E4FD3436}">
       <text>
         <r>
           <rPr>
@@ -658,7 +1043,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D36" authorId="0" shapeId="0" xr:uid="{90457D58-D5A2-4BFF-925F-DD280FFED479}">
+    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{90457D58-D5A2-4BFF-925F-DD280FFED479}">
       <text>
         <r>
           <rPr>
@@ -672,7 +1057,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D37" authorId="0" shapeId="0" xr:uid="{DE2E0716-78AE-4DAF-B782-6F59EBF63292}">
+    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{DE2E0716-78AE-4DAF-B782-6F59EBF63292}">
       <text>
         <r>
           <rPr>
@@ -683,391 +1068,6 @@
             <scheme val="minor"/>
           </rPr>
           <t>Built from the publisher's standard URL pattern; not opened directly - please spot-check. Real Decreto 266/2021 (MOVES III), BOE-A-2021-5869 of 14.04.2021 (ID and date confirmed on BOE).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D38" authorId="0" shapeId="0" xr:uid="{F5FAC7D6-CC6A-42C1-85BF-0C07B000E395}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Final updated NECP 2021-2030 (Aug 2024), English. German version: same link with _de.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D39" authorId="0" shapeId="0" xr:uid="{A632FA71-FAA3-4976-992D-9EF4E5E18B0A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Consolidated EEG 2023 (gesetze-im-internet.de). Same URL as earlier PDF column.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D40" authorId="0" shapeId="0" xr:uid="{D15C6D15-094B-48F6-B3CE-83EA83899870}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Enacted law, BGBl. 2024 I Nr. 151 (in force 16.05.2024). Replaces the BMWK summary as the policy document.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D41" authorId="0" shapeId="0" xr:uid="{7C6248C4-6F1B-4E76-AFFF-E9E0F8A106A7}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Enacted law, BGBl. 2023 I Nr. 133 (22.05.2023). Verified scan of the same gazette: https://epflicht.ulb.uni-bonn.de/download/pdf/775275</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D42" authorId="0" shapeId="0" xr:uid="{4F270FE6-455D-475A-AF90-E3D41CF0EDB6}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Consolidated EnWG.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D43" authorId="0" shapeId="0" xr:uid="{89F84E70-4A97-4E38-A1F5-8126A7485411}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Consolidated text valid from 22.05.2026 (Bezirksregierung Arnsberg).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D44" authorId="0" shapeId="0" xr:uid="{280662A7-29A5-45BA-A25C-73321C94BB18}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Original act of 12.06.2024 (REVOSax). Note: amended 10.09.2025; consolidated HTML at revosax.sachsen.de/vorschrift/20864.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D45" authorId="0" shapeId="0" xr:uid="{C2F9E7CD-E4A6-42E7-A852-76AC8FBC95C1}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. NOTE: this is the NEW BüGembeteilG M-V (GVOBl. 28.04.2026) that replaced the 2016 law named in the row. No official PDF of the 2016 original was found.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D46" authorId="0" shapeId="0" xr:uid="{0BA27891-D32B-413B-ACB5-8BDE169AD307}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. GVBl. I Nr. 30/2019. Law repealed 28.11.2025, replaced by BbgEESG (GVBl. I Nr. 26/2025): https://www.landesrecht.brandenburg.de/dislservice/public/disl/dokumente/11224/dokument/16894</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D47" authorId="0" shapeId="0" xr:uid="{10E51489-0262-4624-95FB-7A7493528561}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Final updated NECP (Oct 2024), English. Hungarian: same link with _hu.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D48" authorId="0" shapeId="0" xr:uid="{94F4788C-50B8-44DF-965B-8091418C0D6B}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>No direct PDF of the KEHOP Plusz programme document could be found (palyazat.gov.hu serves it through a script-rendered page). Left blank rather than linking a web page.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D49" authorId="0" shapeId="0" xr:uid="{6D7AB778-5E38-47A9-89F5-22C44BF7DDCD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Magyar Közlöny 2017/168 containing Govt. Decree 299/2017 (X.17.), p. 28304. Download link returns the PDF.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D50" authorId="0" shapeId="0" xr:uid="{86010D8A-3BEA-4CD8-A4F4-C99ED974FD9E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>NKFIH 'palyazati-felhivas' URLs serve the call PDF directly (confirmed on other NKFIH calls). Call 2020-3.1.4-ZFR-EKM.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{91740555-7138-43AE-BD55-DCF9D57639BD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Call document, 2nd amendment (06.08.2024).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D52" authorId="0" shapeId="0" xr:uid="{29510604-14BD-43BE-954E-BB95DC972A75}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. EU BUILD UP one-stop-shop factsheet on RenoPont. RenoPont is NGO-run; no government policy document exists.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D53" authorId="0" shapeId="0" xr:uid="{51A0B6B0-FFC5-4C3E-86CF-140CB3AFB436}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Magyar Közlöny 2023/171 containing Govt. Decree 518/2023 (XI.30.), p. 9279. Housing loan scheme, not an energy policy.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D54" authorId="0" shapeId="0" xr:uid="{15CB8238-AEC9-4B69-AF7C-8E0934754DEE}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Final updated NECP (July 2024).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D55" authorId="0" shapeId="0" xr:uid="{7A2A96C3-B4FC-407E-AF23-794618E674FB}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. CAP25 main report (latest published; CAP26 not yet out).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D56" authorId="0" shapeId="0" xr:uid="{C427DF66-A7EB-4B82-90F1-A0E846EB4237}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. DECC 'Micro-generation Support Scheme (MSS)' final scheme design document.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D57" authorId="0" shapeId="0" xr:uid="{662152E2-17AB-47A3-97D7-33B0035F98B5}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. SEAI Solar PV Grant Application Guide (scheme rules).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D58" authorId="0" shapeId="0" xr:uid="{EACBCA3C-2180-4B23-B822-8BA759744D3E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. SRESS 1 Application Information Pack. The separate T&amp;Cs PDF link could not be located; the pack references them.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D59" authorId="0" shapeId="0" xr:uid="{620DC488-411D-4173-B7A5-435D11ADA902}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Better Energy Homes Application Guide incl. Terms &amp; Conditions.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D60" authorId="0" shapeId="0" xr:uid="{DB12F6EB-AC19-4206-ABF1-4B90BEC67AEF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. T&amp;Cs v2.0, Sept 2024.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D61" authorId="0" shapeId="0" xr:uid="{E61E0C92-6990-4A34-83ED-011972D3A1A9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Communities Energy Grant guidelines, 2024 call.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D62" authorId="0" shapeId="0" xr:uid="{336FF0D6-B0F1-49C3-831E-91C277F19D39}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>PNIEC 2024 final (MASE). Same URL as earlier PDF column.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{D68A8417-5A26-416D-9919-2280443B3569}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. GU n.285 of 30.11.2021, S.O. n.42 (original text). Consolidated copy (non-official host): https://faolex.fao.org/docs/pdf/ita227896.pdf</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D64" authorId="0" shapeId="0" xr:uid="{CCA3A71E-DAC3-40A7-BB94-06C0DEA5A180}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>MASE document-library link that serves the PDF of DM 7.12.2023 n.414 (CACER decree), published 23.01.2024.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D65" authorId="0" shapeId="0" xr:uid="{26635959-3244-4949-9FCA-F023FA659D8A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>MASE document-library PDF: CACER Operational Rules (July 2025) governing the PNRR 40% grant.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D66" authorId="0" shapeId="0" xr:uid="{59826D51-C97C-48E9-9AE4-71DCD3DE2A9A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Ordinanza n.24 of 30.06.2022 approving the CER call.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D67" authorId="0" shapeId="0" xr:uid="{E64F13D7-23E9-44AB-B844-53DE8D0A3D34}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Representative: Piedmont Regional Law 12/2018 (first regional CER law).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D68" authorId="0" shapeId="0" xr:uid="{310119CF-5582-4958-A35D-19CF0F7A8C9A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 as published (DR 1st series n.10, pp.3-185). A copy of the same file is at https://ordemdosengenheiros.pt/fotos/especialidades/0000300185_19938915836571aac8a132c.pdf</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D69" authorId="0" shapeId="0" xr:uid="{73160079-E26A-486A-96C1-0BCE740FAD4E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 (energy communities incl. cooperative form). Same document as REC framework row.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D70" authorId="0" shapeId="0" xr:uid="{01751E51-B477-4058-9F90-57799D92504C}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Regulation of the Programa de Apoio a Edifícios Mais Sustentáveis (Despacho 8745/2020). NON-OFFICIAL host (municipality); the official DR PDF could not be located.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D71" authorId="0" shapeId="0" xr:uid="{EF14530C-C227-49F0-98BE-9079397A86E7}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Direct PDF link found in search results. Lei 12/2022 (State Budget 2022) that added item 2.37 to VAT List I. Reportedly expired 30.06.2025.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D72" authorId="0" shapeId="0" xr:uid="{915BDAC7-735F-42D4-A53B-97B55CF2EABB}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <rFont val="Carlito"/>
-          </rPr>
-          <t>Built from the publisher's standard PDF URL pattern (pattern confirmed on other documents); not opened directly - please spot-check. Decree-Law 15/2022 (self-consumption/UPAC rules). Same document as REC framework row.</t>
         </r>
       </text>
     </comment>
@@ -1164,7 +1164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="155">
   <si>
     <t>Federal funding for energy-efficient buildings (BEG)</t>
   </si>
@@ -1262,9 +1262,6 @@
     <t>https://www.seai.ie/sites/default/files/grants/home-energy-grants/fully-funded-upgrades-for-eligible-homes/SCHEME-GUIDELINES.pdf</t>
   </si>
   <si>
-    <t>https://seai.ie/grants/community-grants/project-criteria-and-funding/CEG-Guidelines-2024.pdf</t>
-  </si>
-  <si>
     <t>https://assets.gov.ie/static/documents/Climate_Action_Plan_2025_updated_cover.pdf</t>
   </si>
   <si>
@@ -1277,9 +1274,6 @@
     <t>https://docs.italia.it/media/pdf/strategia-nazionale-competenze-digitali-docs/1.0/strategia-nazionale-competenze-digitali-docs.pdf</t>
   </si>
   <si>
-    <t>https://www.apren.pt/contents/legislation/decreto-legislativo-regional-17-2025-a.pdf</t>
-  </si>
-  <si>
     <t>https://www.miteco.gob.es/content/dam/miteco/es/prensa/estrategianacionalcontralapobrezaenergetica2019-2024_tcm30-496282.pdf</t>
   </si>
   <si>
@@ -1319,9 +1313,6 @@
     <t>https://vizmuvek.hu/files/public/new/torvenyek-jogszabalyok/2023-_evi_ciii-_torv-ny-kozlonyallapot-20231222.pdf</t>
   </si>
   <si>
-    <t>https://www.rtb.ie/images/uploads/Comms%20and%20Research/Housing_for_All.pdf</t>
-  </si>
-  <si>
     <t>https://www.gazzettaufficiale.it/eli/gu/2020/05/19/128/so/21/sg/pdf</t>
   </si>
   <si>
@@ -1479,15 +1470,6 @@
   </si>
   <si>
     <t>https://www.gesetze-im-internet.de/eeg_2014/EEG_2023.pdf</t>
-  </si>
-  <si>
-    <t>https://www.recht.bund.de/bgbl/1/2024/151/regelungstext.pdf</t>
-  </si>
-  <si>
-    <t>https://www.recht.bund.de/bgbl/1/2023/133/regelungstext.pdf</t>
-  </si>
-  <si>
-    <t>https://revosax.sachsen.de/vorschrift_gesamt/20863/47088.pdf</t>
   </si>
   <si>
     <t>https://www.regierung-mv.de/static/Regierungsportal/Justizministerium/Inhalte/Rechtliches/GVOBI.M-V/GVOBl.%20Nr.%2012%20v.%2028.4.2026.pdf</t>
@@ -1653,6 +1635,12 @@
   </si>
   <si>
     <t>Restriction of freight traffic, urban logistics, and tourist vehicle traffic</t>
+  </si>
+  <si>
+    <t>https://www.recht.bund.de/bgbl/1/2023/133/regelungstext.pdf?__blob=publicationFile&amp;v=1</t>
+  </si>
+  <si>
+    <t>https://www.recht.bund.de/bgbl/1/2024/151/regelungstext.pdf?__blob=publicationFile&amp;v=1</t>
   </si>
 </sst>
 </file>
@@ -2023,22 +2011,22 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" t="s">
-        <v>42</v>
-      </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2049,16 +2037,16 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
         <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H2">
         <f>LEN(C2)</f>
@@ -2076,13 +2064,13 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H64" si="0">LEN(C3)</f>
@@ -2097,16 +2085,16 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H4">
         <f t="shared" si="0"/>
@@ -2127,10 +2115,10 @@
         <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
@@ -2148,13 +2136,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
@@ -2172,13 +2160,13 @@
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
@@ -2193,16 +2181,16 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H8">
         <f t="shared" si="0"/>
@@ -2220,13 +2208,13 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H9">
         <f t="shared" si="0"/>
@@ -2235,610 +2223,586 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>147</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
-        <v>139</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>62</v>
+        <v>137</v>
+      </c>
+      <c r="F10" t="s">
+        <v>131</v>
       </c>
       <c r="H10">
         <f t="shared" ref="H10" si="1">LEN(C10)</f>
-        <v>77</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>147</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="E11" t="s">
-        <v>139</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>62</v>
+        <v>132</v>
+      </c>
+      <c r="F11" t="s">
+        <v>131</v>
       </c>
       <c r="H11">
         <f t="shared" si="0"/>
-        <v>77</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>148</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>154</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>62</v>
+        <v>132</v>
+      </c>
+      <c r="F12" t="s">
+        <v>131</v>
       </c>
       <c r="H12">
         <f t="shared" si="0"/>
-        <v>65</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
         <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>153</v>
       </c>
       <c r="E13" t="s">
-        <v>139</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>62</v>
+        <v>132</v>
+      </c>
+      <c r="F13" t="s">
+        <v>131</v>
       </c>
       <c r="H13">
         <f t="shared" si="0"/>
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>132</v>
+      </c>
+      <c r="F14" t="s">
+        <v>131</v>
       </c>
       <c r="H14">
         <f t="shared" si="0"/>
-        <v>70</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
         <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>151</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="E15" t="s">
-        <v>139</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>62</v>
+        <v>132</v>
+      </c>
+      <c r="F15" t="s">
+        <v>131</v>
       </c>
       <c r="H15">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" t="s">
-        <v>143</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
+      </c>
+      <c r="F16" t="s">
+        <v>131</v>
       </c>
       <c r="H16">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="E17" t="s">
-        <v>143</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>62</v>
+        <v>132</v>
+      </c>
+      <c r="F17" t="s">
+        <v>131</v>
       </c>
       <c r="H17">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
       </c>
       <c r="C18" t="s">
-        <v>2</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
+      </c>
+      <c r="D18" t="s">
+        <v>103</v>
+      </c>
+      <c r="E18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F18" t="s">
+        <v>131</v>
       </c>
       <c r="H18">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H19">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E20" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H20">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>142</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="E21" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H21">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D22" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E22" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H22">
         <f t="shared" si="0"/>
-        <v>93</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s">
-        <v>52</v>
-      </c>
-      <c r="E23" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H23">
         <f t="shared" si="0"/>
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
         <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="D24" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E24" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H24">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s">
         <v>19</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="D25" t="s">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>62</v>
+        <v>137</v>
+      </c>
+      <c r="F25" t="s">
+        <v>131</v>
       </c>
       <c r="H25">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
         <v>19</v>
       </c>
       <c r="C26" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" t="s">
-        <v>141</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>62</v>
+        <v>69</v>
+      </c>
+      <c r="F26" t="s">
+        <v>131</v>
       </c>
       <c r="H26">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
         <v>19</v>
       </c>
       <c r="C27" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="E27" t="s">
-        <v>141</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>62</v>
+        <v>133</v>
+      </c>
+      <c r="F27" t="s">
+        <v>131</v>
       </c>
       <c r="H27">
         <f t="shared" si="0"/>
-        <v>58</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C28" t="s">
-        <v>154</v>
+        <v>71</v>
       </c>
       <c r="D28" t="s">
-        <v>54</v>
+        <v>106</v>
       </c>
       <c r="E28" t="s">
-        <v>141</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>62</v>
+        <v>133</v>
+      </c>
+      <c r="F28" t="s">
+        <v>131</v>
       </c>
       <c r="H28">
         <f t="shared" si="0"/>
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15" customHeight="1">
       <c r="A29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" t="s">
+        <v>107</v>
+      </c>
+      <c r="E29" t="s">
+        <v>133</v>
+      </c>
+      <c r="F29" t="s">
+        <v>131</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="0"/>
         <v>24</v>
-      </c>
-      <c r="B29" t="s">
-        <v>22</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" t="s">
-        <v>55</v>
-      </c>
-      <c r="E29" t="s">
-        <v>141</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H29">
-        <f t="shared" si="0"/>
-        <v>116</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="17.5" customHeight="1">
       <c r="A30" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>155</v>
+        <v>19</v>
+      </c>
+      <c r="C30" t="s">
+        <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>108</v>
       </c>
       <c r="E30" t="s">
-        <v>141</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>62</v>
+        <v>137</v>
+      </c>
+      <c r="F30" t="s">
+        <v>131</v>
       </c>
       <c r="H30">
         <f t="shared" si="0"/>
-        <v>97</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>156</v>
+        <v>74</v>
       </c>
       <c r="D31" t="s">
-        <v>36</v>
+        <v>109</v>
       </c>
       <c r="E31" t="s">
-        <v>141</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>62</v>
+        <v>133</v>
+      </c>
+      <c r="F31" t="s">
+        <v>131</v>
       </c>
       <c r="H31">
         <f t="shared" si="0"/>
-        <v>71</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C32" t="s">
-        <v>157</v>
+        <v>6</v>
       </c>
       <c r="D32" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="E32" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H32">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B33" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="0"/>
         <v>22</v>
-      </c>
-      <c r="C33" t="s">
-        <v>158</v>
-      </c>
-      <c r="D33" t="s">
-        <v>57</v>
-      </c>
-      <c r="E33" t="s">
-        <v>141</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H33">
-        <f t="shared" si="0"/>
-        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B34" t="s">
         <v>19</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" t="s">
-        <v>37</v>
-      </c>
-      <c r="E34" t="s">
-        <v>140</v>
+        <v>2</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H34">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" t="s">
-        <v>38</v>
-      </c>
-      <c r="E35" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H35">
         <f t="shared" si="0"/>
@@ -2847,70 +2811,70 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D36" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E36" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H36">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B37" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E37" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H37">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B38" t="s">
         <v>19</v>
       </c>
       <c r="C38" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D38" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E38" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F38" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H38">
         <f t="shared" si="0"/>
@@ -2919,481 +2883,481 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B39" t="s">
         <v>19</v>
       </c>
       <c r="C39" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>104</v>
+        <v>32</v>
       </c>
       <c r="E39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H39">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B40" t="s">
         <v>19</v>
       </c>
       <c r="C40" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D40" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H40">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B41" t="s">
         <v>19</v>
       </c>
       <c r="C41" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D41" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E41" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H41">
         <f t="shared" si="0"/>
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B42" t="s">
         <v>19</v>
       </c>
       <c r="C42" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="D42" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="E42" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F42" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H42">
         <f t="shared" si="0"/>
-        <v>31</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B43" t="s">
         <v>19</v>
       </c>
       <c r="C43" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>114</v>
       </c>
       <c r="E43" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F43" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H43">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
         <v>19</v>
       </c>
       <c r="C44" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D44" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F44" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H44">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B45" t="s">
         <v>19</v>
       </c>
       <c r="C45" t="s">
-        <v>70</v>
-      </c>
-      <c r="D45" t="s">
-        <v>108</v>
-      </c>
-      <c r="E45" t="s">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="F45" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H45">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B46" t="s">
         <v>19</v>
       </c>
       <c r="C46" t="s">
-        <v>71</v>
+        <v>147</v>
       </c>
       <c r="D46" t="s">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="E46" t="s">
-        <v>138</v>
-      </c>
-      <c r="F46" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H46">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B47" t="s">
         <v>19</v>
       </c>
       <c r="C47" t="s">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="D47" t="s">
-        <v>110</v>
+        <v>49</v>
       </c>
       <c r="E47" t="s">
-        <v>143</v>
-      </c>
-      <c r="F47" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H47">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B48" t="s">
         <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>72</v>
-      </c>
-      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" t="s">
+        <v>50</v>
+      </c>
+      <c r="E48" t="s">
         <v>137</v>
       </c>
+      <c r="F48" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="H48">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B49" t="s">
         <v>19</v>
       </c>
       <c r="C49" t="s">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="D49" t="s">
-        <v>111</v>
+        <v>34</v>
       </c>
       <c r="E49" t="s">
-        <v>139</v>
-      </c>
-      <c r="F49" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H49">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>53</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B50" t="s">
         <v>19</v>
       </c>
       <c r="C50" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="D50" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="E50" t="s">
-        <v>139</v>
-      </c>
-      <c r="F50" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H50">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B51" t="s">
         <v>19</v>
       </c>
       <c r="C51" t="s">
-        <v>75</v>
+        <v>17</v>
       </c>
       <c r="D51" t="s">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="E51" t="s">
-        <v>139</v>
-      </c>
-      <c r="F51" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H51">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B52" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C52" t="s">
-        <v>76</v>
+        <v>148</v>
       </c>
       <c r="D52" t="s">
-        <v>114</v>
+        <v>51</v>
       </c>
       <c r="E52" t="s">
-        <v>143</v>
-      </c>
-      <c r="F52" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H52">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>62</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B53" t="s">
-        <v>19</v>
-      </c>
-      <c r="C53" t="s">
-        <v>77</v>
+        <v>22</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>138</v>
       </c>
       <c r="D53" t="s">
-        <v>115</v>
+        <v>52</v>
       </c>
       <c r="E53" t="s">
-        <v>139</v>
-      </c>
-      <c r="F53" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H53">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>116</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
-      </c>
-      <c r="C54" t="s">
-        <v>63</v>
+        <v>22</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="D54" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="E54" t="s">
-        <v>143</v>
-      </c>
-      <c r="F54" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H54">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B55" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C55" t="s">
-        <v>78</v>
+        <v>150</v>
       </c>
       <c r="D55" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E55" t="s">
-        <v>143</v>
-      </c>
-      <c r="F55" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H55">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>71</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B56" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C56" t="s">
-        <v>79</v>
+        <v>151</v>
       </c>
       <c r="D56" t="s">
-        <v>117</v>
+        <v>54</v>
       </c>
       <c r="E56" t="s">
-        <v>143</v>
-      </c>
-      <c r="F56" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H56">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>61</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B57" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="D57" t="s">
-        <v>118</v>
+        <v>54</v>
       </c>
       <c r="E57" t="s">
-        <v>143</v>
-      </c>
-      <c r="F57" t="s">
-        <v>137</v>
+        <v>135</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H57">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B58" t="s">
         <v>19</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D58" t="s">
-        <v>119</v>
+        <v>34</v>
       </c>
       <c r="E58" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F58" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H58">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B59" t="s">
         <v>19</v>
@@ -3402,22 +3366,22 @@
         <v>82</v>
       </c>
       <c r="D59" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E59" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F59" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H59">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B60" t="s">
         <v>19</v>
@@ -3426,22 +3390,22 @@
         <v>83</v>
       </c>
       <c r="D60" t="s">
-        <v>121</v>
+        <v>33</v>
       </c>
       <c r="E60" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F60" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H60">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B61" t="s">
         <v>19</v>
@@ -3450,17 +3414,17 @@
         <v>84</v>
       </c>
       <c r="D61" t="s">
-        <v>32</v>
+        <v>117</v>
       </c>
       <c r="E61" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="F61" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H61">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -3471,20 +3435,20 @@
         <v>19</v>
       </c>
       <c r="C62" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="D62" t="s">
-        <v>35</v>
+        <v>118</v>
       </c>
       <c r="E62" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F62" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H62">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -3495,49 +3459,43 @@
         <v>19</v>
       </c>
       <c r="C63" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D63" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E63" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F63" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H63">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B64" t="s">
         <v>19</v>
       </c>
       <c r="C64" t="s">
-        <v>86</v>
-      </c>
-      <c r="D64" t="s">
-        <v>34</v>
-      </c>
-      <c r="E64" t="s">
-        <v>141</v>
-      </c>
-      <c r="F64" t="s">
-        <v>137</v>
+        <v>5</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H64">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B65" t="s">
         <v>19</v>
@@ -3546,22 +3504,22 @@
         <v>87</v>
       </c>
       <c r="D65" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E65" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F65" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H65">
         <f t="shared" ref="H65:H80" si="2">LEN(C65)</f>
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B66" t="s">
         <v>19</v>
@@ -3570,22 +3528,22 @@
         <v>88</v>
       </c>
       <c r="D66" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E66" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F66" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H66">
         <f t="shared" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B67" t="s">
         <v>19</v>
@@ -3594,17 +3552,17 @@
         <v>89</v>
       </c>
       <c r="D67" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E67" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F67" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H67">
         <f t="shared" si="2"/>
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -3618,17 +3576,17 @@
         <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E68" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F68" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H68">
         <f t="shared" si="2"/>
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -3642,89 +3600,89 @@
         <v>91</v>
       </c>
       <c r="D69" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F69" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H69">
         <f t="shared" si="2"/>
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B70" t="s">
         <v>19</v>
       </c>
       <c r="C70" t="s">
-        <v>92</v>
+        <v>9</v>
       </c>
       <c r="D70" t="s">
-        <v>127</v>
+        <v>36</v>
       </c>
       <c r="E70" t="s">
-        <v>140</v>
-      </c>
-      <c r="F70" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H70">
         <f t="shared" si="2"/>
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B71" t="s">
         <v>19</v>
       </c>
       <c r="C71" t="s">
-        <v>93</v>
+        <v>8</v>
       </c>
       <c r="D71" t="s">
-        <v>128</v>
+        <v>37</v>
       </c>
       <c r="E71" t="s">
-        <v>140</v>
-      </c>
-      <c r="F71" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H71">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>16</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B72" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C72" t="s">
-        <v>94</v>
+        <v>7</v>
       </c>
       <c r="D72" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
       <c r="E72" t="s">
-        <v>140</v>
-      </c>
-      <c r="F72" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="H72">
         <f t="shared" si="2"/>
-        <v>29</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -3735,16 +3693,16 @@
         <v>19</v>
       </c>
       <c r="C73" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D73" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E73" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F73" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H73">
         <f t="shared" si="2"/>
@@ -3759,16 +3717,16 @@
         <v>19</v>
       </c>
       <c r="C74" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D74" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E74" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F74" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H74">
         <f t="shared" si="2"/>
@@ -3783,16 +3741,16 @@
         <v>19</v>
       </c>
       <c r="C75" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D75" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E75" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F75" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H75">
         <f t="shared" si="2"/>
@@ -3807,16 +3765,16 @@
         <v>19</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D76" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E76" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F76" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H76">
         <f t="shared" si="2"/>
@@ -3831,16 +3789,16 @@
         <v>19</v>
       </c>
       <c r="C77" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D77" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E77" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F77" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H77">
         <f t="shared" si="2"/>
@@ -3855,16 +3813,16 @@
         <v>19</v>
       </c>
       <c r="C78" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D78" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E78" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F78" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H78">
         <f t="shared" si="2"/>
@@ -3879,16 +3837,16 @@
         <v>19</v>
       </c>
       <c r="C79" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D79" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E79" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F79" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H79">
         <f t="shared" si="2"/>
@@ -3903,16 +3861,16 @@
         <v>19</v>
       </c>
       <c r="C80" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D80" t="s">
+        <v>130</v>
+      </c>
+      <c r="E80" t="s">
         <v>136</v>
       </c>
-      <c r="E80" t="s">
-        <v>142</v>
-      </c>
       <c r="F80" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H80">
         <f t="shared" si="2"/>
@@ -3920,6 +3878,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F80" xr:uid="{A7C53CE1-AB1B-4F69-8A65-C29313BFC2AD}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F80">
+      <sortCondition ref="A1:A80"/>
+    </sortState>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{FA16102E-24DC-48CF-AC71-D68C5E17A565}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{F04BE974-3F1B-4744-A8FA-D6E3C80DFA8A}"/>
@@ -3929,76 +3892,69 @@
     <hyperlink ref="D7" r:id="rId6" xr:uid="{FD7B5D66-ED3B-4DC8-AF7D-320FB8B8DCF0}"/>
     <hyperlink ref="D8" r:id="rId7" xr:uid="{014A4358-20DF-4B5F-AE9F-C26FE89E87A9}"/>
     <hyperlink ref="D9" r:id="rId8" xr:uid="{2BBA6949-C4A4-42E3-BEA4-ABD14D852388}"/>
-    <hyperlink ref="D11" r:id="rId9" xr:uid="{97BAEC4D-7419-45F2-8D16-CB115B0CB032}"/>
-    <hyperlink ref="D16" r:id="rId10" xr:uid="{BA89AC2D-6F7A-4FD2-976D-42C1F35A4FE6}"/>
-    <hyperlink ref="D17" r:id="rId11" xr:uid="{2E124691-8A80-401A-802C-2F82A366E356}"/>
-    <hyperlink ref="D19" r:id="rId12" xr:uid="{644586B2-493A-453E-9F85-0C756A72F1C8}"/>
-    <hyperlink ref="D20" r:id="rId13" xr:uid="{D991AF5E-1724-496F-8731-5209CC5CB261}"/>
-    <hyperlink ref="D21" r:id="rId14" xr:uid="{A894FC6B-F122-4CF3-86DC-BDCA0737F2B0}"/>
-    <hyperlink ref="D22" r:id="rId15" xr:uid="{E1DEE2A9-7080-48F2-8499-B3F200C5E387}"/>
-    <hyperlink ref="D23" r:id="rId16" xr:uid="{4E433208-4F67-4949-9BF2-FDBDA35728D4}"/>
-    <hyperlink ref="D24" r:id="rId17" xr:uid="{0DC7D7A9-9ABA-421C-8ACB-61E96F26C589}"/>
-    <hyperlink ref="D25" r:id="rId18" xr:uid="{FFEF1E00-7C49-412F-9191-A6E2D4FD22A9}"/>
-    <hyperlink ref="D26" r:id="rId19" xr:uid="{BD4B5AA3-6373-4484-9CC8-2794F6CED241}"/>
-    <hyperlink ref="D27" r:id="rId20" xr:uid="{8B6E0311-A3FD-4221-B3EE-18443B4F4070}"/>
-    <hyperlink ref="D28" r:id="rId21" xr:uid="{05F631B4-D997-4A49-A861-D5119FCEBA08}"/>
-    <hyperlink ref="D29" r:id="rId22" xr:uid="{197D6BD6-6D24-433F-B21E-D04EE9054948}"/>
-    <hyperlink ref="D30" r:id="rId23" xr:uid="{72F68369-A900-4BD1-8990-8564783A8C3C}"/>
-    <hyperlink ref="D31" r:id="rId24" xr:uid="{69CD499B-1F3C-4502-99D0-575B484A534B}"/>
-    <hyperlink ref="D32" r:id="rId25" xr:uid="{6F2DAF87-0E2E-4FDB-84E9-CFDE14FFBFFF}"/>
-    <hyperlink ref="D33" r:id="rId26" xr:uid="{2CCAC871-D236-408B-B9FA-D2EB1D5E0C40}"/>
-    <hyperlink ref="D34" r:id="rId27" xr:uid="{428F6EA1-5818-4A51-BC68-3325CF77C295}"/>
-    <hyperlink ref="D35" r:id="rId28" xr:uid="{F1AFAC85-C328-421F-B5C4-2A236B4C7B84}"/>
-    <hyperlink ref="D36" r:id="rId29" xr:uid="{2929F43F-FF43-4F43-966D-B25524FC9841}"/>
-    <hyperlink ref="D37" r:id="rId30" xr:uid="{0D6A551E-F4F1-4374-9482-B1FB082B2BB4}"/>
-    <hyperlink ref="D38" r:id="rId31" xr:uid="{2756696F-298F-48A9-A14D-59F28D76A4B3}"/>
-    <hyperlink ref="D39" r:id="rId32" xr:uid="{DFA6C174-E909-4E02-97D7-ECF69BCEDC04}"/>
-    <hyperlink ref="D40" r:id="rId33" xr:uid="{42975378-F8C7-40C1-8FD9-279140112DB9}"/>
-    <hyperlink ref="D41" r:id="rId34" xr:uid="{9E861439-53A3-4E94-84A9-77B02FA0DF14}"/>
-    <hyperlink ref="D42" r:id="rId35" xr:uid="{94B7F12E-4A8A-4908-B754-CD6440105814}"/>
-    <hyperlink ref="D43" r:id="rId36" xr:uid="{D37203B1-3467-4791-97C1-D5FA4916FA26}"/>
-    <hyperlink ref="D44" r:id="rId37" xr:uid="{69F21018-CAF9-40D4-9B96-319BAB603A08}"/>
-    <hyperlink ref="D45" r:id="rId38" xr:uid="{6223FD59-6F2A-4FD8-B03E-F896BAFD2C13}"/>
-    <hyperlink ref="D46" r:id="rId39" xr:uid="{88661935-A581-4BF7-890D-E123AA21750F}"/>
-    <hyperlink ref="D47" r:id="rId40" xr:uid="{C93170FF-369B-4F8C-9D4F-3DB5C4DFF48A}"/>
-    <hyperlink ref="D49" r:id="rId41" xr:uid="{8A27131A-644F-48E1-9CB2-A067DA0D2C07}"/>
-    <hyperlink ref="D50" r:id="rId42" xr:uid="{65F1E7A9-ABA4-4FA3-8EC1-C5D350DE5FC7}"/>
-    <hyperlink ref="D51" r:id="rId43" xr:uid="{A1B0C38E-8D5F-4F6A-BE8A-B3A5C46C63F4}"/>
-    <hyperlink ref="D52" r:id="rId44" xr:uid="{4E616770-2491-4BA8-8304-F1402698BAA5}"/>
-    <hyperlink ref="D53" r:id="rId45" xr:uid="{3499484E-3B42-45C9-8CFD-55B5209AAEFB}"/>
-    <hyperlink ref="D54" r:id="rId46" xr:uid="{9587478C-75BB-4F66-AD7C-259631A01D5C}"/>
-    <hyperlink ref="D55" r:id="rId47" xr:uid="{9DB31D3B-4EF9-4EE0-8C38-17699E60A181}"/>
-    <hyperlink ref="D56" r:id="rId48" xr:uid="{B579180D-B0D5-4902-AC7E-5AAE895B8E58}"/>
-    <hyperlink ref="D57" r:id="rId49" xr:uid="{5EDACE02-0B6F-4168-B759-B80CD83049AF}"/>
-    <hyperlink ref="D58" r:id="rId50" xr:uid="{384922C9-A261-4069-8457-03FCDDC44FA2}"/>
-    <hyperlink ref="D59" r:id="rId51" xr:uid="{927A1F11-1DBA-4D32-96EE-DEA5B84C9A5D}"/>
-    <hyperlink ref="D60" r:id="rId52" xr:uid="{5D0D0DB8-AD46-4986-9B98-EAFB83433CDE}"/>
-    <hyperlink ref="D61" r:id="rId53" xr:uid="{9F0FFF7E-5E5B-4DA5-8208-87705FF0163C}"/>
-    <hyperlink ref="D62" r:id="rId54" xr:uid="{37BC9865-D94E-40FA-8D37-2EFA79072828}"/>
-    <hyperlink ref="D63" r:id="rId55" xr:uid="{913102AD-B2A9-4932-AC1D-9F71D34FBB0E}"/>
-    <hyperlink ref="D64" r:id="rId56" xr:uid="{D1CC8E83-9106-4779-B44D-BB84D924B760}"/>
-    <hyperlink ref="D65" r:id="rId57" xr:uid="{8844F135-685E-44D1-9D60-7468AD8DB244}"/>
-    <hyperlink ref="D66" r:id="rId58" xr:uid="{7B93DFA0-0E83-439A-BD2A-1414A9F63FCC}"/>
-    <hyperlink ref="D67" r:id="rId59" xr:uid="{89BFE053-4D54-4309-872E-5BEC8034683F}"/>
-    <hyperlink ref="D68" r:id="rId60" xr:uid="{D435E386-9058-438B-BA38-2873D56361D3}"/>
-    <hyperlink ref="D69" r:id="rId61" xr:uid="{9C4D4F21-640D-4DC9-952F-49248A1DBB25}"/>
-    <hyperlink ref="D70" r:id="rId62" xr:uid="{D36E8947-16AE-4484-9C63-D3E87960D04A}"/>
-    <hyperlink ref="D71" r:id="rId63" xr:uid="{F18510CB-AFA0-4AF6-8336-235F88E914E9}"/>
-    <hyperlink ref="D72" r:id="rId64" xr:uid="{7BD00D44-3373-4BFB-BFAC-64857BD433BB}"/>
-    <hyperlink ref="D73" r:id="rId65" xr:uid="{86A4FAB7-787E-49CA-A931-19A0CBAF06A8}"/>
-    <hyperlink ref="D74" r:id="rId66" xr:uid="{3AAE6721-3155-45D9-8E86-006C9F2E7837}"/>
-    <hyperlink ref="D75" r:id="rId67" xr:uid="{E33DAA04-E7BD-4CA8-8C7A-38532E177F9A}"/>
-    <hyperlink ref="D76" r:id="rId68" xr:uid="{5C3E49A6-5C26-4786-9FAB-879E0846C84D}"/>
-    <hyperlink ref="D77" r:id="rId69" xr:uid="{18540A14-49D4-4368-B1B7-DB16D1659669}"/>
-    <hyperlink ref="D78" r:id="rId70" xr:uid="{D0654701-E81D-454A-B6FF-255E627E169D}"/>
-    <hyperlink ref="D79" r:id="rId71" xr:uid="{2345F39C-F6B3-4540-900C-5E8B6C7D2510}"/>
-    <hyperlink ref="D80" r:id="rId72" xr:uid="{782EEC21-1F26-48AE-83A1-75F8799B7570}"/>
-    <hyperlink ref="D13" r:id="rId73" xr:uid="{75903415-E398-48EF-85AA-576F7EFD4BFD}"/>
-    <hyperlink ref="D12" r:id="rId74" xr:uid="{4A12E92D-D5E7-4C58-832D-CEA3CB8B359C}"/>
-    <hyperlink ref="D15" r:id="rId75" xr:uid="{B68D5E7F-5EE4-493D-980F-0F27D52CCD80}"/>
-    <hyperlink ref="D10" r:id="rId76" xr:uid="{E324A0A9-1119-4732-BCBF-35505542BD54}"/>
+    <hyperlink ref="D20" r:id="rId9" xr:uid="{97BAEC4D-7419-45F2-8D16-CB115B0CB032}"/>
+    <hyperlink ref="D32" r:id="rId10" xr:uid="{BA89AC2D-6F7A-4FD2-976D-42C1F35A4FE6}"/>
+    <hyperlink ref="D36" r:id="rId11" xr:uid="{D991AF5E-1724-496F-8731-5209CC5CB261}"/>
+    <hyperlink ref="D37" r:id="rId12" xr:uid="{A894FC6B-F122-4CF3-86DC-BDCA0737F2B0}"/>
+    <hyperlink ref="D46" r:id="rId13" xr:uid="{E1DEE2A9-7080-48F2-8499-B3F200C5E387}"/>
+    <hyperlink ref="D47" r:id="rId14" xr:uid="{4E433208-4F67-4949-9BF2-FDBDA35728D4}"/>
+    <hyperlink ref="D48" r:id="rId15" xr:uid="{0DC7D7A9-9ABA-421C-8ACB-61E96F26C589}"/>
+    <hyperlink ref="D49" r:id="rId16" xr:uid="{FFEF1E00-7C49-412F-9191-A6E2D4FD22A9}"/>
+    <hyperlink ref="D50" r:id="rId17" xr:uid="{BD4B5AA3-6373-4484-9CC8-2794F6CED241}"/>
+    <hyperlink ref="D51" r:id="rId18" xr:uid="{8B6E0311-A3FD-4221-B3EE-18443B4F4070}"/>
+    <hyperlink ref="D52" r:id="rId19" xr:uid="{05F631B4-D997-4A49-A861-D5119FCEBA08}"/>
+    <hyperlink ref="D53" r:id="rId20" xr:uid="{197D6BD6-6D24-433F-B21E-D04EE9054948}"/>
+    <hyperlink ref="D54" r:id="rId21" xr:uid="{72F68369-A900-4BD1-8990-8564783A8C3C}"/>
+    <hyperlink ref="D55" r:id="rId22" xr:uid="{69CD499B-1F3C-4502-99D0-575B484A534B}"/>
+    <hyperlink ref="D56" r:id="rId23" xr:uid="{6F2DAF87-0E2E-4FDB-84E9-CFDE14FFBFFF}"/>
+    <hyperlink ref="D57" r:id="rId24" xr:uid="{2CCAC871-D236-408B-B9FA-D2EB1D5E0C40}"/>
+    <hyperlink ref="D70" r:id="rId25" xr:uid="{F1AFAC85-C328-421F-B5C4-2A236B4C7B84}"/>
+    <hyperlink ref="D71" r:id="rId26" xr:uid="{2929F43F-FF43-4F43-966D-B25524FC9841}"/>
+    <hyperlink ref="D72" r:id="rId27" xr:uid="{0D6A551E-F4F1-4374-9482-B1FB082B2BB4}"/>
+    <hyperlink ref="D10" r:id="rId28" xr:uid="{2756696F-298F-48A9-A14D-59F28D76A4B3}"/>
+    <hyperlink ref="D11" r:id="rId29" xr:uid="{DFA6C174-E909-4E02-97D7-ECF69BCEDC04}"/>
+    <hyperlink ref="D14" r:id="rId30" xr:uid="{94B7F12E-4A8A-4908-B754-CD6440105814}"/>
+    <hyperlink ref="D15" r:id="rId31" xr:uid="{D37203B1-3467-4791-97C1-D5FA4916FA26}"/>
+    <hyperlink ref="D17" r:id="rId32" xr:uid="{6223FD59-6F2A-4FD8-B03E-F896BAFD2C13}"/>
+    <hyperlink ref="D18" r:id="rId33" xr:uid="{88661935-A581-4BF7-890D-E123AA21750F}"/>
+    <hyperlink ref="D25" r:id="rId34" xr:uid="{C93170FF-369B-4F8C-9D4F-3DB5C4DFF48A}"/>
+    <hyperlink ref="D27" r:id="rId35" xr:uid="{8A27131A-644F-48E1-9CB2-A067DA0D2C07}"/>
+    <hyperlink ref="D28" r:id="rId36" xr:uid="{65F1E7A9-ABA4-4FA3-8EC1-C5D350DE5FC7}"/>
+    <hyperlink ref="D29" r:id="rId37" xr:uid="{A1B0C38E-8D5F-4F6A-BE8A-B3A5C46C63F4}"/>
+    <hyperlink ref="D30" r:id="rId38" xr:uid="{4E616770-2491-4BA8-8304-F1402698BAA5}"/>
+    <hyperlink ref="D31" r:id="rId39" xr:uid="{3499484E-3B42-45C9-8CFD-55B5209AAEFB}"/>
+    <hyperlink ref="D38" r:id="rId40" xr:uid="{9587478C-75BB-4F66-AD7C-259631A01D5C}"/>
+    <hyperlink ref="D39" r:id="rId41" xr:uid="{9DB31D3B-4EF9-4EE0-8C38-17699E60A181}"/>
+    <hyperlink ref="D40" r:id="rId42" xr:uid="{B579180D-B0D5-4902-AC7E-5AAE895B8E58}"/>
+    <hyperlink ref="D41" r:id="rId43" xr:uid="{5EDACE02-0B6F-4168-B759-B80CD83049AF}"/>
+    <hyperlink ref="D42" r:id="rId44" xr:uid="{384922C9-A261-4069-8457-03FCDDC44FA2}"/>
+    <hyperlink ref="D43" r:id="rId45" xr:uid="{927A1F11-1DBA-4D32-96EE-DEA5B84C9A5D}"/>
+    <hyperlink ref="D44" r:id="rId46" xr:uid="{5D0D0DB8-AD46-4986-9B98-EAFB83433CDE}"/>
+    <hyperlink ref="D58" r:id="rId47" xr:uid="{37BC9865-D94E-40FA-8D37-2EFA79072828}"/>
+    <hyperlink ref="D59" r:id="rId48" xr:uid="{913102AD-B2A9-4932-AC1D-9F71D34FBB0E}"/>
+    <hyperlink ref="D60" r:id="rId49" xr:uid="{D1CC8E83-9106-4779-B44D-BB84D924B760}"/>
+    <hyperlink ref="D61" r:id="rId50" xr:uid="{8844F135-685E-44D1-9D60-7468AD8DB244}"/>
+    <hyperlink ref="D62" r:id="rId51" xr:uid="{7B93DFA0-0E83-439A-BD2A-1414A9F63FCC}"/>
+    <hyperlink ref="D63" r:id="rId52" xr:uid="{89BFE053-4D54-4309-872E-5BEC8034683F}"/>
+    <hyperlink ref="D65" r:id="rId53" xr:uid="{D435E386-9058-438B-BA38-2873D56361D3}"/>
+    <hyperlink ref="D66" r:id="rId54" xr:uid="{9C4D4F21-640D-4DC9-952F-49248A1DBB25}"/>
+    <hyperlink ref="D67" r:id="rId55" xr:uid="{D36E8947-16AE-4484-9C63-D3E87960D04A}"/>
+    <hyperlink ref="D68" r:id="rId56" xr:uid="{F18510CB-AFA0-4AF6-8336-235F88E914E9}"/>
+    <hyperlink ref="D69" r:id="rId57" xr:uid="{7BD00D44-3373-4BFB-BFAC-64857BD433BB}"/>
+    <hyperlink ref="D73" r:id="rId58" xr:uid="{86A4FAB7-787E-49CA-A931-19A0CBAF06A8}"/>
+    <hyperlink ref="D74" r:id="rId59" xr:uid="{3AAE6721-3155-45D9-8E86-006C9F2E7837}"/>
+    <hyperlink ref="D75" r:id="rId60" xr:uid="{E33DAA04-E7BD-4CA8-8C7A-38532E177F9A}"/>
+    <hyperlink ref="D76" r:id="rId61" xr:uid="{5C3E49A6-5C26-4786-9FAB-879E0846C84D}"/>
+    <hyperlink ref="D77" r:id="rId62" xr:uid="{18540A14-49D4-4368-B1B7-DB16D1659669}"/>
+    <hyperlink ref="D78" r:id="rId63" xr:uid="{D0654701-E81D-454A-B6FF-255E627E169D}"/>
+    <hyperlink ref="D79" r:id="rId64" xr:uid="{2345F39C-F6B3-4540-900C-5E8B6C7D2510}"/>
+    <hyperlink ref="D80" r:id="rId65" xr:uid="{782EEC21-1F26-48AE-83A1-75F8799B7570}"/>
+    <hyperlink ref="D22" r:id="rId66" xr:uid="{75903415-E398-48EF-85AA-576F7EFD4BFD}"/>
+    <hyperlink ref="D21" r:id="rId67" xr:uid="{4A12E92D-D5E7-4C58-832D-CEA3CB8B359C}"/>
+    <hyperlink ref="D24" r:id="rId68" xr:uid="{B68D5E7F-5EE4-493D-980F-0F27D52CCD80}"/>
+    <hyperlink ref="D19" r:id="rId69" xr:uid="{E324A0A9-1119-4732-BCBF-35505542BD54}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId77"/>
+  <legacyDrawing r:id="rId70"/>
 </worksheet>
 </file>
</xml_diff>